<commit_message>
Poprawki do badań i protokołów
</commit_message>
<xml_diff>
--- a/app/templates/protocol_template.xlsx
+++ b/app/templates/protocol_template.xlsx
@@ -1798,7 +1798,7 @@
   <dimension ref="B1:BN71"/>
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="3" width="2.109375" customWidth="1"/>
     <col min="4" max="17" width="1.77734375" customWidth="1"/>
     <col min="18" max="23" width="1.6640625" customWidth="1"/>
@@ -7677,7 +7677,7 @@
     <mergeCell ref="B64:M64"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0" footer="0"/>
+  <pageMargins left="0.19685039370078741" right="0.65622539370078736" top="0.31496062992125984" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="90" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>

<commit_message>
poprawki protokołów do 16 zawodników
</commit_message>
<xml_diff>
--- a/app/templates/protocol_template.xlsx
+++ b/app/templates/protocol_template.xlsx
@@ -16,7 +16,7 @@
     <sheet name="protokół" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">protokół!$A$1:$BH$71</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">protokół!$A$1:$BH$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1811,7 +1811,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{067EC097-671F-4825-B7F3-5CC1B353F4A8}">
   <sheetPr codeName="Arkusz1"/>
-  <dimension ref="B1:BN71"/>
+  <dimension ref="B1:BN67"/>
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="2.88671875" customWidth="1"/>
@@ -2534,7 +2534,7 @@
       <c r="BG10" s="117"/>
       <c r="BH10" s="118"/>
     </row>
-    <row r="11" spans="2:62">
+    <row r="11" spans="2:62" ht="14.85" customHeight="1">
       <c r="B11" s="84"/>
       <c r="C11" s="73"/>
       <c r="D11" s="148"/>
@@ -2600,7 +2600,7 @@
       <c r="BH11" s="118"/>
       <c r="BJ11" s="11"/>
     </row>
-    <row r="12" spans="2:62">
+    <row r="12" spans="2:62" ht="14.85" customHeight="1">
       <c r="B12" s="36"/>
       <c r="C12" s="110"/>
       <c r="D12" s="148"/>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="BH12" s="29"/>
     </row>
-    <row r="13" spans="2:62">
+    <row r="13" spans="2:62" ht="14.85" customHeight="1">
       <c r="B13" s="36"/>
       <c r="C13" s="110"/>
       <c r="D13" s="148"/>
@@ -2738,7 +2738,7 @@
       <c r="BG13" s="30"/>
       <c r="BH13" s="31"/>
     </row>
-    <row r="14" spans="2:62">
+    <row r="14" spans="2:62" ht="14.85" customHeight="1">
       <c r="B14" s="36"/>
       <c r="C14" s="110"/>
       <c r="D14" s="148"/>
@@ -2799,7 +2799,7 @@
       <c r="BG14" s="32"/>
       <c r="BH14" s="33"/>
     </row>
-    <row r="15" spans="2:62">
+    <row r="15" spans="2:62" ht="14.85" customHeight="1">
       <c r="B15" s="36"/>
       <c r="C15" s="110"/>
       <c r="D15" s="148"/>
@@ -2864,7 +2864,7 @@
       <c r="BG15" s="71"/>
       <c r="BH15" s="72"/>
     </row>
-    <row r="16" spans="2:62">
+    <row r="16" spans="2:62" ht="14.85" customHeight="1">
       <c r="B16" s="36"/>
       <c r="C16" s="110"/>
       <c r="D16" s="148"/>
@@ -2929,7 +2929,7 @@
       <c r="BG16" s="76"/>
       <c r="BH16" s="72"/>
     </row>
-    <row r="17" spans="2:60">
+    <row r="17" spans="2:60" ht="14.85" customHeight="1">
       <c r="B17" s="36"/>
       <c r="C17" s="110"/>
       <c r="D17" s="148"/>
@@ -2994,7 +2994,7 @@
       <c r="BG17" s="71"/>
       <c r="BH17" s="72"/>
     </row>
-    <row r="18" spans="2:60">
+    <row r="18" spans="2:60" ht="14.85" customHeight="1">
       <c r="B18" s="36"/>
       <c r="C18" s="110"/>
       <c r="D18" s="148"/>
@@ -3059,7 +3059,7 @@
       <c r="BG18" s="71"/>
       <c r="BH18" s="72"/>
     </row>
-    <row r="19" spans="2:60">
+    <row r="19" spans="2:60" ht="14.85" customHeight="1">
       <c r="B19" s="36"/>
       <c r="C19" s="110"/>
       <c r="D19" s="148"/>
@@ -3124,7 +3124,7 @@
       <c r="BG19" s="71"/>
       <c r="BH19" s="72"/>
     </row>
-    <row r="20" spans="2:60">
+    <row r="20" spans="2:60" ht="14.85" customHeight="1">
       <c r="B20" s="36"/>
       <c r="C20" s="110"/>
       <c r="D20" s="148"/>
@@ -3189,7 +3189,7 @@
       <c r="BG20" s="71"/>
       <c r="BH20" s="72"/>
     </row>
-    <row r="21" spans="2:60">
+    <row r="21" spans="2:60" ht="14.85" customHeight="1">
       <c r="B21" s="36"/>
       <c r="C21" s="110"/>
       <c r="D21" s="148"/>
@@ -3254,7 +3254,7 @@
       <c r="BG21" s="71"/>
       <c r="BH21" s="72"/>
     </row>
-    <row r="22" spans="2:60">
+    <row r="22" spans="2:60" ht="14.85" customHeight="1">
       <c r="B22" s="36"/>
       <c r="C22" s="110"/>
       <c r="D22" s="148"/>
@@ -3319,7 +3319,7 @@
       <c r="BG22" s="71"/>
       <c r="BH22" s="72"/>
     </row>
-    <row r="23" spans="2:60">
+    <row r="23" spans="2:60" ht="14.85" customHeight="1">
       <c r="B23" s="36"/>
       <c r="C23" s="110"/>
       <c r="D23" s="148"/>
@@ -3384,7 +3384,7 @@
       <c r="BG23" s="71"/>
       <c r="BH23" s="72"/>
     </row>
-    <row r="24" spans="2:60">
+    <row r="24" spans="2:60" ht="14.85" customHeight="1">
       <c r="B24" s="36"/>
       <c r="C24" s="110"/>
       <c r="D24" s="148"/>
@@ -3449,7 +3449,7 @@
       <c r="BG24" s="71"/>
       <c r="BH24" s="72"/>
     </row>
-    <row r="25" spans="2:60">
+    <row r="25" spans="2:60" ht="14.85" customHeight="1">
       <c r="B25" s="36"/>
       <c r="C25" s="110"/>
       <c r="D25" s="148"/>
@@ -3514,7 +3514,7 @@
       <c r="BG25" s="71"/>
       <c r="BH25" s="72"/>
     </row>
-    <row r="26" spans="2:60">
+    <row r="26" spans="2:60" ht="14.85" customHeight="1">
       <c r="B26" s="36"/>
       <c r="C26" s="110"/>
       <c r="D26" s="148"/>
@@ -3579,44 +3579,54 @@
       <c r="BG26" s="71"/>
       <c r="BH26" s="72"/>
     </row>
-    <row r="27" spans="2:60">
-      <c r="B27" s="36"/>
-      <c r="C27" s="110"/>
-      <c r="D27" s="148"/>
-      <c r="E27" s="149"/>
-      <c r="F27" s="149"/>
-      <c r="G27" s="149"/>
-      <c r="H27" s="149"/>
-      <c r="I27" s="149"/>
-      <c r="J27" s="149"/>
-      <c r="K27" s="149"/>
-      <c r="L27" s="149"/>
-      <c r="M27" s="149"/>
-      <c r="N27" s="149"/>
-      <c r="O27" s="149"/>
-      <c r="P27" s="149"/>
-      <c r="Q27" s="150"/>
-      <c r="R27" s="132"/>
-      <c r="S27" s="133"/>
-      <c r="T27" s="132"/>
-      <c r="U27" s="133"/>
-      <c r="V27" s="78"/>
-      <c r="W27" s="80"/>
-      <c r="X27" s="78"/>
-      <c r="Y27" s="79"/>
-      <c r="Z27" s="80"/>
-      <c r="AA27" s="78"/>
-      <c r="AB27" s="79"/>
-      <c r="AC27" s="80"/>
-      <c r="AD27" s="78"/>
-      <c r="AE27" s="79"/>
-      <c r="AF27" s="80"/>
-      <c r="AG27" s="78"/>
-      <c r="AH27" s="79"/>
-      <c r="AI27" s="80"/>
-      <c r="AJ27" s="78"/>
-      <c r="AK27" s="79"/>
-      <c r="AL27" s="80"/>
+    <row r="27" spans="2:60" ht="13.2" customHeight="1">
+      <c r="B27" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="158"/>
+      <c r="D27" s="158"/>
+      <c r="E27" s="158"/>
+      <c r="F27" s="158"/>
+      <c r="G27" s="159"/>
+      <c r="H27" s="159"/>
+      <c r="I27" s="159"/>
+      <c r="J27" s="160"/>
+      <c r="K27" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L27" s="124"/>
+      <c r="M27" s="124"/>
+      <c r="N27" s="124"/>
+      <c r="O27" s="124"/>
+      <c r="P27" s="124"/>
+      <c r="Q27" s="125"/>
+      <c r="R27" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="S27" s="129"/>
+      <c r="T27" s="129"/>
+      <c r="U27" s="129"/>
+      <c r="V27" s="129"/>
+      <c r="W27" s="129"/>
+      <c r="X27" s="130"/>
+      <c r="Y27" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z27" s="129"/>
+      <c r="AA27" s="129"/>
+      <c r="AB27" s="129"/>
+      <c r="AC27" s="129"/>
+      <c r="AD27" s="129"/>
+      <c r="AE27" s="130"/>
+      <c r="AF27" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AG27" s="124"/>
+      <c r="AH27" s="124"/>
+      <c r="AI27" s="124"/>
+      <c r="AJ27" s="124"/>
+      <c r="AK27" s="124"/>
+      <c r="AL27" s="125"/>
       <c r="AM27" s="36"/>
       <c r="AN27" s="73"/>
       <c r="AO27" s="76"/>
@@ -3644,310 +3654,310 @@
       <c r="BG27" s="71"/>
       <c r="BH27" s="72"/>
     </row>
-    <row r="28" spans="2:60">
-      <c r="B28" s="36"/>
-      <c r="C28" s="110"/>
-      <c r="D28" s="148"/>
-      <c r="E28" s="149"/>
-      <c r="F28" s="149"/>
-      <c r="G28" s="149"/>
-      <c r="H28" s="149"/>
-      <c r="I28" s="149"/>
-      <c r="J28" s="149"/>
-      <c r="K28" s="149"/>
-      <c r="L28" s="149"/>
-      <c r="M28" s="149"/>
-      <c r="N28" s="149"/>
-      <c r="O28" s="149"/>
-      <c r="P28" s="149"/>
-      <c r="Q28" s="150"/>
-      <c r="R28" s="132"/>
-      <c r="S28" s="133"/>
-      <c r="T28" s="132"/>
-      <c r="U28" s="133"/>
-      <c r="V28" s="78"/>
-      <c r="W28" s="80"/>
-      <c r="X28" s="78"/>
-      <c r="Y28" s="79"/>
-      <c r="Z28" s="80"/>
-      <c r="AA28" s="78"/>
-      <c r="AB28" s="79"/>
-      <c r="AC28" s="80"/>
-      <c r="AD28" s="78"/>
-      <c r="AE28" s="79"/>
-      <c r="AF28" s="80"/>
-      <c r="AG28" s="78"/>
-      <c r="AH28" s="79"/>
-      <c r="AI28" s="80"/>
-      <c r="AJ28" s="78"/>
-      <c r="AK28" s="79"/>
-      <c r="AL28" s="80"/>
-      <c r="AM28" s="36"/>
-      <c r="AN28" s="73"/>
-      <c r="AO28" s="76"/>
-      <c r="AP28" s="72"/>
-      <c r="AQ28" s="131"/>
-      <c r="AR28" s="27"/>
-      <c r="AS28" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT28" s="85"/>
-      <c r="AU28" s="86"/>
-      <c r="AV28" s="71"/>
-      <c r="AW28" s="72"/>
-      <c r="AX28" s="84"/>
-      <c r="AY28" s="73"/>
-      <c r="AZ28" s="71"/>
-      <c r="BA28" s="72"/>
-      <c r="BB28" s="26"/>
-      <c r="BC28" s="27"/>
-      <c r="BD28" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE28" s="85"/>
-      <c r="BF28" s="86"/>
-      <c r="BG28" s="71"/>
-      <c r="BH28" s="72"/>
+    <row r="28" spans="2:60" ht="6.6" customHeight="1">
+      <c r="B28" s="151"/>
+      <c r="C28" s="152"/>
+      <c r="D28" s="152"/>
+      <c r="E28" s="152"/>
+      <c r="F28" s="152"/>
+      <c r="G28" s="161"/>
+      <c r="H28" s="161"/>
+      <c r="I28" s="161"/>
+      <c r="J28" s="162"/>
+      <c r="K28" s="175"/>
+      <c r="L28" s="176"/>
+      <c r="M28" s="176"/>
+      <c r="N28" s="176"/>
+      <c r="O28" s="176"/>
+      <c r="P28" s="176"/>
+      <c r="Q28" s="177"/>
+      <c r="R28" s="175"/>
+      <c r="S28" s="176"/>
+      <c r="T28" s="176"/>
+      <c r="U28" s="176"/>
+      <c r="V28" s="176"/>
+      <c r="W28" s="176"/>
+      <c r="X28" s="177"/>
+      <c r="Y28" s="175"/>
+      <c r="Z28" s="176"/>
+      <c r="AA28" s="176"/>
+      <c r="AB28" s="176"/>
+      <c r="AC28" s="176"/>
+      <c r="AD28" s="176"/>
+      <c r="AE28" s="177"/>
+      <c r="AF28" s="175"/>
+      <c r="AG28" s="176"/>
+      <c r="AH28" s="176"/>
+      <c r="AI28" s="176"/>
+      <c r="AJ28" s="176"/>
+      <c r="AK28" s="176"/>
+      <c r="AL28" s="177"/>
+      <c r="AM28" s="187"/>
+      <c r="AN28" s="188"/>
+      <c r="AO28" s="191"/>
+      <c r="AP28" s="192"/>
+      <c r="AQ28" s="191"/>
+      <c r="AR28" s="195"/>
+      <c r="AS28" s="197" t="s">
+        <v>5</v>
+      </c>
+      <c r="AT28" s="199"/>
+      <c r="AU28" s="200"/>
+      <c r="AV28" s="203"/>
+      <c r="AW28" s="200"/>
+      <c r="AX28" s="205"/>
+      <c r="AY28" s="206"/>
+      <c r="AZ28" s="203"/>
+      <c r="BA28" s="200"/>
+      <c r="BB28" s="203"/>
+      <c r="BC28" s="199"/>
+      <c r="BD28" s="197" t="s">
+        <v>5</v>
+      </c>
+      <c r="BE28" s="199"/>
+      <c r="BF28" s="200"/>
+      <c r="BG28" s="203"/>
+      <c r="BH28" s="200"/>
     </row>
-    <row r="29" spans="2:60" ht="13.2" customHeight="1">
-      <c r="B29" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C29" s="158"/>
-      <c r="D29" s="158"/>
-      <c r="E29" s="158"/>
-      <c r="F29" s="158"/>
-      <c r="G29" s="159"/>
-      <c r="H29" s="159"/>
-      <c r="I29" s="159"/>
-      <c r="J29" s="160"/>
-      <c r="K29" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L29" s="124"/>
-      <c r="M29" s="124"/>
-      <c r="N29" s="124"/>
-      <c r="O29" s="124"/>
-      <c r="P29" s="124"/>
-      <c r="Q29" s="125"/>
-      <c r="R29" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="S29" s="129"/>
-      <c r="T29" s="129"/>
-      <c r="U29" s="129"/>
-      <c r="V29" s="129"/>
-      <c r="W29" s="129"/>
-      <c r="X29" s="130"/>
-      <c r="Y29" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="Z29" s="129"/>
-      <c r="AA29" s="129"/>
-      <c r="AB29" s="129"/>
-      <c r="AC29" s="129"/>
-      <c r="AD29" s="129"/>
-      <c r="AE29" s="130"/>
-      <c r="AF29" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="AG29" s="124"/>
-      <c r="AH29" s="124"/>
-      <c r="AI29" s="124"/>
-      <c r="AJ29" s="124"/>
-      <c r="AK29" s="124"/>
-      <c r="AL29" s="125"/>
-      <c r="AM29" s="36"/>
-      <c r="AN29" s="73"/>
-      <c r="AO29" s="76"/>
-      <c r="AP29" s="72"/>
-      <c r="AQ29" s="131"/>
-      <c r="AR29" s="27"/>
-      <c r="AS29" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT29" s="85"/>
-      <c r="AU29" s="86"/>
-      <c r="AV29" s="71"/>
-      <c r="AW29" s="72"/>
-      <c r="AX29" s="84"/>
-      <c r="AY29" s="73"/>
-      <c r="AZ29" s="71"/>
-      <c r="BA29" s="72"/>
-      <c r="BB29" s="26"/>
-      <c r="BC29" s="27"/>
-      <c r="BD29" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE29" s="85"/>
-      <c r="BF29" s="86"/>
-      <c r="BG29" s="71"/>
-      <c r="BH29" s="72"/>
+    <row r="29" spans="2:60" ht="6.6" customHeight="1">
+      <c r="B29" s="153"/>
+      <c r="C29" s="154"/>
+      <c r="D29" s="154"/>
+      <c r="E29" s="154"/>
+      <c r="F29" s="154"/>
+      <c r="G29" s="161"/>
+      <c r="H29" s="161"/>
+      <c r="I29" s="161"/>
+      <c r="J29" s="162"/>
+      <c r="K29" s="126"/>
+      <c r="L29" s="127"/>
+      <c r="M29" s="127"/>
+      <c r="N29" s="127"/>
+      <c r="O29" s="127"/>
+      <c r="P29" s="127"/>
+      <c r="Q29" s="128"/>
+      <c r="R29" s="126"/>
+      <c r="S29" s="127"/>
+      <c r="T29" s="127"/>
+      <c r="U29" s="127"/>
+      <c r="V29" s="127"/>
+      <c r="W29" s="127"/>
+      <c r="X29" s="128"/>
+      <c r="Y29" s="126"/>
+      <c r="Z29" s="127"/>
+      <c r="AA29" s="127"/>
+      <c r="AB29" s="127"/>
+      <c r="AC29" s="127"/>
+      <c r="AD29" s="127"/>
+      <c r="AE29" s="128"/>
+      <c r="AF29" s="126"/>
+      <c r="AG29" s="127"/>
+      <c r="AH29" s="127"/>
+      <c r="AI29" s="127"/>
+      <c r="AJ29" s="127"/>
+      <c r="AK29" s="127"/>
+      <c r="AL29" s="128"/>
+      <c r="AM29" s="189"/>
+      <c r="AN29" s="190"/>
+      <c r="AO29" s="193"/>
+      <c r="AP29" s="194"/>
+      <c r="AQ29" s="193"/>
+      <c r="AR29" s="196"/>
+      <c r="AS29" s="198"/>
+      <c r="AT29" s="201"/>
+      <c r="AU29" s="202"/>
+      <c r="AV29" s="204"/>
+      <c r="AW29" s="202"/>
+      <c r="AX29" s="207"/>
+      <c r="AY29" s="208"/>
+      <c r="AZ29" s="204"/>
+      <c r="BA29" s="202"/>
+      <c r="BB29" s="204"/>
+      <c r="BC29" s="201"/>
+      <c r="BD29" s="198"/>
+      <c r="BE29" s="201"/>
+      <c r="BF29" s="202"/>
+      <c r="BG29" s="204"/>
+      <c r="BH29" s="202"/>
     </row>
-    <row r="30" spans="2:60" ht="6.6" customHeight="1">
-      <c r="B30" s="151"/>
-      <c r="C30" s="152"/>
-      <c r="D30" s="152"/>
-      <c r="E30" s="152"/>
-      <c r="F30" s="152"/>
-      <c r="G30" s="161"/>
-      <c r="H30" s="161"/>
-      <c r="I30" s="161"/>
-      <c r="J30" s="162"/>
-      <c r="K30" s="175"/>
-      <c r="L30" s="176"/>
-      <c r="M30" s="176"/>
-      <c r="N30" s="176"/>
-      <c r="O30" s="176"/>
-      <c r="P30" s="176"/>
-      <c r="Q30" s="177"/>
-      <c r="R30" s="175"/>
-      <c r="S30" s="176"/>
-      <c r="T30" s="176"/>
-      <c r="U30" s="176"/>
-      <c r="V30" s="176"/>
-      <c r="W30" s="176"/>
-      <c r="X30" s="177"/>
-      <c r="Y30" s="175"/>
-      <c r="Z30" s="176"/>
-      <c r="AA30" s="176"/>
-      <c r="AB30" s="176"/>
-      <c r="AC30" s="176"/>
-      <c r="AD30" s="176"/>
-      <c r="AE30" s="177"/>
-      <c r="AF30" s="175"/>
-      <c r="AG30" s="176"/>
-      <c r="AH30" s="176"/>
-      <c r="AI30" s="176"/>
-      <c r="AJ30" s="176"/>
-      <c r="AK30" s="176"/>
-      <c r="AL30" s="177"/>
-      <c r="AM30" s="187"/>
-      <c r="AN30" s="188"/>
-      <c r="AO30" s="191"/>
-      <c r="AP30" s="192"/>
-      <c r="AQ30" s="191"/>
-      <c r="AR30" s="195"/>
-      <c r="AS30" s="197" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT30" s="199"/>
-      <c r="AU30" s="200"/>
-      <c r="AV30" s="203"/>
-      <c r="AW30" s="200"/>
-      <c r="AX30" s="205"/>
-      <c r="AY30" s="206"/>
-      <c r="AZ30" s="203"/>
-      <c r="BA30" s="200"/>
-      <c r="BB30" s="203"/>
-      <c r="BC30" s="199"/>
-      <c r="BD30" s="197" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE30" s="199"/>
-      <c r="BF30" s="200"/>
-      <c r="BG30" s="203"/>
-      <c r="BH30" s="200"/>
+    <row r="30" spans="2:60">
+      <c r="B30" s="163"/>
+      <c r="C30" s="164"/>
+      <c r="D30" s="164"/>
+      <c r="E30" s="164"/>
+      <c r="F30" s="164"/>
+      <c r="G30" s="164"/>
+      <c r="H30" s="164"/>
+      <c r="I30" s="164"/>
+      <c r="J30" s="165"/>
+      <c r="K30" s="157"/>
+      <c r="L30" s="155"/>
+      <c r="M30" s="155"/>
+      <c r="N30" s="155"/>
+      <c r="O30" s="155"/>
+      <c r="P30" s="155"/>
+      <c r="Q30" s="156"/>
+      <c r="R30" s="157"/>
+      <c r="S30" s="155"/>
+      <c r="T30" s="155"/>
+      <c r="U30" s="155"/>
+      <c r="V30" s="155"/>
+      <c r="W30" s="155"/>
+      <c r="X30" s="156"/>
+      <c r="Y30" s="157"/>
+      <c r="Z30" s="155"/>
+      <c r="AA30" s="155"/>
+      <c r="AB30" s="155"/>
+      <c r="AC30" s="155"/>
+      <c r="AD30" s="155"/>
+      <c r="AE30" s="156"/>
+      <c r="AF30" s="157"/>
+      <c r="AG30" s="155"/>
+      <c r="AH30" s="155"/>
+      <c r="AI30" s="155"/>
+      <c r="AJ30" s="155"/>
+      <c r="AK30" s="155"/>
+      <c r="AL30" s="156"/>
+      <c r="AM30" s="84"/>
+      <c r="AN30" s="73"/>
+      <c r="AO30" s="71"/>
+      <c r="AP30" s="72"/>
+      <c r="AQ30" s="26"/>
+      <c r="AR30" s="27"/>
+      <c r="AS30" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="AT30" s="85"/>
+      <c r="AU30" s="86"/>
+      <c r="AV30" s="71"/>
+      <c r="AW30" s="72"/>
+      <c r="AX30" s="84"/>
+      <c r="AY30" s="73"/>
+      <c r="AZ30" s="71"/>
+      <c r="BA30" s="72"/>
+      <c r="BB30" s="26"/>
+      <c r="BC30" s="27"/>
+      <c r="BD30" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="BE30" s="85"/>
+      <c r="BF30" s="86"/>
+      <c r="BG30" s="71"/>
+      <c r="BH30" s="72"/>
     </row>
-    <row r="31" spans="2:60" ht="6.6" customHeight="1">
-      <c r="B31" s="153"/>
-      <c r="C31" s="154"/>
-      <c r="D31" s="154"/>
-      <c r="E31" s="154"/>
-      <c r="F31" s="154"/>
-      <c r="G31" s="161"/>
-      <c r="H31" s="161"/>
-      <c r="I31" s="161"/>
-      <c r="J31" s="162"/>
-      <c r="K31" s="126"/>
-      <c r="L31" s="127"/>
-      <c r="M31" s="127"/>
-      <c r="N31" s="127"/>
-      <c r="O31" s="127"/>
-      <c r="P31" s="127"/>
-      <c r="Q31" s="128"/>
-      <c r="R31" s="126"/>
-      <c r="S31" s="127"/>
-      <c r="T31" s="127"/>
-      <c r="U31" s="127"/>
-      <c r="V31" s="127"/>
-      <c r="W31" s="127"/>
-      <c r="X31" s="128"/>
-      <c r="Y31" s="126"/>
-      <c r="Z31" s="127"/>
-      <c r="AA31" s="127"/>
-      <c r="AB31" s="127"/>
-      <c r="AC31" s="127"/>
-      <c r="AD31" s="127"/>
-      <c r="AE31" s="128"/>
-      <c r="AF31" s="126"/>
-      <c r="AG31" s="127"/>
-      <c r="AH31" s="127"/>
-      <c r="AI31" s="127"/>
-      <c r="AJ31" s="127"/>
-      <c r="AK31" s="127"/>
-      <c r="AL31" s="128"/>
-      <c r="AM31" s="189"/>
-      <c r="AN31" s="190"/>
-      <c r="AO31" s="193"/>
-      <c r="AP31" s="194"/>
-      <c r="AQ31" s="193"/>
-      <c r="AR31" s="196"/>
-      <c r="AS31" s="198"/>
-      <c r="AT31" s="201"/>
-      <c r="AU31" s="202"/>
-      <c r="AV31" s="204"/>
-      <c r="AW31" s="202"/>
-      <c r="AX31" s="207"/>
-      <c r="AY31" s="208"/>
-      <c r="AZ31" s="204"/>
-      <c r="BA31" s="202"/>
-      <c r="BB31" s="204"/>
-      <c r="BC31" s="201"/>
-      <c r="BD31" s="198"/>
-      <c r="BE31" s="201"/>
-      <c r="BF31" s="202"/>
-      <c r="BG31" s="204"/>
-      <c r="BH31" s="202"/>
+    <row r="31" spans="2:60">
+      <c r="B31" s="166" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="167"/>
+      <c r="D31" s="167"/>
+      <c r="E31" s="167"/>
+      <c r="F31" s="167"/>
+      <c r="G31" s="167"/>
+      <c r="H31" s="167"/>
+      <c r="I31" s="167"/>
+      <c r="J31" s="168"/>
+      <c r="K31" s="166" t="s">
+        <v>26</v>
+      </c>
+      <c r="L31" s="167"/>
+      <c r="M31" s="167"/>
+      <c r="N31" s="167"/>
+      <c r="O31" s="167"/>
+      <c r="P31" s="167"/>
+      <c r="Q31" s="168"/>
+      <c r="R31" s="166" t="s">
+        <v>26</v>
+      </c>
+      <c r="S31" s="167"/>
+      <c r="T31" s="167"/>
+      <c r="U31" s="167"/>
+      <c r="V31" s="167"/>
+      <c r="W31" s="167"/>
+      <c r="X31" s="168"/>
+      <c r="Y31" s="166" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z31" s="167"/>
+      <c r="AA31" s="167"/>
+      <c r="AB31" s="167"/>
+      <c r="AC31" s="167"/>
+      <c r="AD31" s="167"/>
+      <c r="AE31" s="168"/>
+      <c r="AF31" s="166" t="s">
+        <v>26</v>
+      </c>
+      <c r="AG31" s="167"/>
+      <c r="AH31" s="167"/>
+      <c r="AI31" s="167"/>
+      <c r="AJ31" s="167"/>
+      <c r="AK31" s="167"/>
+      <c r="AL31" s="168"/>
+      <c r="AM31" s="84"/>
+      <c r="AN31" s="73"/>
+      <c r="AO31" s="71"/>
+      <c r="AP31" s="72"/>
+      <c r="AQ31" s="26"/>
+      <c r="AR31" s="27"/>
+      <c r="AS31" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="AT31" s="85"/>
+      <c r="AU31" s="86"/>
+      <c r="AV31" s="71"/>
+      <c r="AW31" s="72"/>
+      <c r="AX31" s="84"/>
+      <c r="AY31" s="73"/>
+      <c r="AZ31" s="71"/>
+      <c r="BA31" s="72"/>
+      <c r="BB31" s="26"/>
+      <c r="BC31" s="27"/>
+      <c r="BD31" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="BE31" s="85"/>
+      <c r="BF31" s="86"/>
+      <c r="BG31" s="71"/>
+      <c r="BH31" s="72"/>
     </row>
     <row r="32" spans="2:60">
-      <c r="B32" s="163"/>
-      <c r="C32" s="164"/>
-      <c r="D32" s="164"/>
-      <c r="E32" s="164"/>
-      <c r="F32" s="164"/>
-      <c r="G32" s="164"/>
-      <c r="H32" s="164"/>
-      <c r="I32" s="164"/>
-      <c r="J32" s="165"/>
-      <c r="K32" s="157"/>
-      <c r="L32" s="155"/>
-      <c r="M32" s="155"/>
-      <c r="N32" s="155"/>
-      <c r="O32" s="155"/>
-      <c r="P32" s="155"/>
-      <c r="Q32" s="156"/>
-      <c r="R32" s="157"/>
-      <c r="S32" s="155"/>
-      <c r="T32" s="155"/>
-      <c r="U32" s="155"/>
-      <c r="V32" s="155"/>
-      <c r="W32" s="155"/>
-      <c r="X32" s="156"/>
-      <c r="Y32" s="157"/>
-      <c r="Z32" s="155"/>
-      <c r="AA32" s="155"/>
-      <c r="AB32" s="155"/>
-      <c r="AC32" s="155"/>
-      <c r="AD32" s="155"/>
-      <c r="AE32" s="156"/>
-      <c r="AF32" s="157"/>
-      <c r="AG32" s="155"/>
-      <c r="AH32" s="155"/>
-      <c r="AI32" s="155"/>
-      <c r="AJ32" s="155"/>
-      <c r="AK32" s="155"/>
-      <c r="AL32" s="156"/>
+      <c r="B32" s="169"/>
+      <c r="C32" s="170"/>
+      <c r="D32" s="170"/>
+      <c r="E32" s="170"/>
+      <c r="F32" s="170"/>
+      <c r="G32" s="170"/>
+      <c r="H32" s="170"/>
+      <c r="I32" s="170"/>
+      <c r="J32" s="171"/>
+      <c r="K32" s="169"/>
+      <c r="L32" s="170"/>
+      <c r="M32" s="170"/>
+      <c r="N32" s="170"/>
+      <c r="O32" s="170"/>
+      <c r="P32" s="170"/>
+      <c r="Q32" s="171"/>
+      <c r="R32" s="169"/>
+      <c r="S32" s="170"/>
+      <c r="T32" s="170"/>
+      <c r="U32" s="170"/>
+      <c r="V32" s="170"/>
+      <c r="W32" s="170"/>
+      <c r="X32" s="171"/>
+      <c r="Y32" s="169"/>
+      <c r="Z32" s="170"/>
+      <c r="AA32" s="170"/>
+      <c r="AB32" s="170"/>
+      <c r="AC32" s="170"/>
+      <c r="AD32" s="170"/>
+      <c r="AE32" s="171"/>
+      <c r="AF32" s="169"/>
+      <c r="AG32" s="170"/>
+      <c r="AH32" s="170"/>
+      <c r="AI32" s="170"/>
+      <c r="AJ32" s="170"/>
+      <c r="AK32" s="170"/>
+      <c r="AL32" s="171"/>
       <c r="AM32" s="84"/>
       <c r="AN32" s="73"/>
       <c r="AO32" s="71"/>
@@ -3976,53 +3986,50 @@
       <c r="BH32" s="72"/>
     </row>
     <row r="33" spans="2:60">
-      <c r="B33" s="166" t="s">
-        <v>25</v>
-      </c>
-      <c r="C33" s="167"/>
-      <c r="D33" s="167"/>
-      <c r="E33" s="167"/>
-      <c r="F33" s="167"/>
-      <c r="G33" s="167"/>
-      <c r="H33" s="167"/>
-      <c r="I33" s="167"/>
-      <c r="J33" s="168"/>
-      <c r="K33" s="166" t="s">
-        <v>26</v>
-      </c>
-      <c r="L33" s="167"/>
-      <c r="M33" s="167"/>
-      <c r="N33" s="167"/>
-      <c r="O33" s="167"/>
-      <c r="P33" s="167"/>
-      <c r="Q33" s="168"/>
-      <c r="R33" s="166" t="s">
-        <v>26</v>
-      </c>
-      <c r="S33" s="167"/>
-      <c r="T33" s="167"/>
-      <c r="U33" s="167"/>
-      <c r="V33" s="167"/>
-      <c r="W33" s="167"/>
-      <c r="X33" s="168"/>
-      <c r="Y33" s="166" t="s">
-        <v>26</v>
-      </c>
-      <c r="Z33" s="167"/>
-      <c r="AA33" s="167"/>
-      <c r="AB33" s="167"/>
-      <c r="AC33" s="167"/>
-      <c r="AD33" s="167"/>
-      <c r="AE33" s="168"/>
-      <c r="AF33" s="166" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG33" s="167"/>
-      <c r="AH33" s="167"/>
-      <c r="AI33" s="167"/>
-      <c r="AJ33" s="167"/>
-      <c r="AK33" s="167"/>
-      <c r="AL33" s="168"/>
+      <c r="B33" s="107" t="s">
+        <v>27</v>
+      </c>
+      <c r="C33" s="108"/>
+      <c r="D33" s="108"/>
+      <c r="E33" s="146">
+        <f>D7</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="146"/>
+      <c r="G33" s="146"/>
+      <c r="H33" s="146"/>
+      <c r="I33" s="146"/>
+      <c r="J33" s="146"/>
+      <c r="K33" s="146"/>
+      <c r="L33" s="146"/>
+      <c r="M33" s="146"/>
+      <c r="N33" s="146"/>
+      <c r="O33" s="146"/>
+      <c r="P33" s="146"/>
+      <c r="Q33" s="146"/>
+      <c r="R33" s="146"/>
+      <c r="S33" s="146"/>
+      <c r="T33" s="146"/>
+      <c r="U33" s="147"/>
+      <c r="V33" s="87" t="s">
+        <v>19</v>
+      </c>
+      <c r="W33" s="88"/>
+      <c r="X33" s="88"/>
+      <c r="Y33" s="88"/>
+      <c r="Z33" s="88"/>
+      <c r="AA33" s="88"/>
+      <c r="AB33" s="88"/>
+      <c r="AC33" s="88"/>
+      <c r="AD33" s="88"/>
+      <c r="AE33" s="88"/>
+      <c r="AF33" s="88"/>
+      <c r="AG33" s="88"/>
+      <c r="AH33" s="88"/>
+      <c r="AI33" s="88"/>
+      <c r="AJ33" s="88"/>
+      <c r="AK33" s="88"/>
+      <c r="AL33" s="89"/>
       <c r="AM33" s="84"/>
       <c r="AN33" s="73"/>
       <c r="AO33" s="71"/>
@@ -4051,43 +4058,63 @@
       <c r="BH33" s="72"/>
     </row>
     <row r="34" spans="2:60">
-      <c r="B34" s="169"/>
-      <c r="C34" s="170"/>
-      <c r="D34" s="170"/>
-      <c r="E34" s="170"/>
-      <c r="F34" s="170"/>
-      <c r="G34" s="170"/>
-      <c r="H34" s="170"/>
-      <c r="I34" s="170"/>
-      <c r="J34" s="171"/>
-      <c r="K34" s="169"/>
-      <c r="L34" s="170"/>
-      <c r="M34" s="170"/>
-      <c r="N34" s="170"/>
-      <c r="O34" s="170"/>
-      <c r="P34" s="170"/>
-      <c r="Q34" s="171"/>
-      <c r="R34" s="169"/>
-      <c r="S34" s="170"/>
-      <c r="T34" s="170"/>
-      <c r="U34" s="170"/>
-      <c r="V34" s="170"/>
-      <c r="W34" s="170"/>
-      <c r="X34" s="171"/>
-      <c r="Y34" s="169"/>
-      <c r="Z34" s="170"/>
-      <c r="AA34" s="170"/>
-      <c r="AB34" s="170"/>
-      <c r="AC34" s="170"/>
-      <c r="AD34" s="170"/>
-      <c r="AE34" s="171"/>
-      <c r="AF34" s="169"/>
-      <c r="AG34" s="170"/>
-      <c r="AH34" s="170"/>
-      <c r="AI34" s="170"/>
-      <c r="AJ34" s="170"/>
-      <c r="AK34" s="170"/>
-      <c r="AL34" s="171"/>
+      <c r="B34" s="87" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34" s="89"/>
+      <c r="D34" s="87" t="s">
+        <v>22</v>
+      </c>
+      <c r="E34" s="88"/>
+      <c r="F34" s="88"/>
+      <c r="G34" s="88"/>
+      <c r="H34" s="88"/>
+      <c r="I34" s="88"/>
+      <c r="J34" s="88"/>
+      <c r="K34" s="88"/>
+      <c r="L34" s="88"/>
+      <c r="M34" s="88"/>
+      <c r="N34" s="88"/>
+      <c r="O34" s="88"/>
+      <c r="P34" s="88"/>
+      <c r="Q34" s="89"/>
+      <c r="R34" s="87" t="s">
+        <v>14</v>
+      </c>
+      <c r="S34" s="89"/>
+      <c r="T34" s="87" t="s">
+        <v>15</v>
+      </c>
+      <c r="U34" s="89"/>
+      <c r="V34" s="87" t="s">
+        <v>16</v>
+      </c>
+      <c r="W34" s="89"/>
+      <c r="X34" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="Y34" s="88"/>
+      <c r="Z34" s="89"/>
+      <c r="AA34" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="AB34" s="88"/>
+      <c r="AC34" s="89"/>
+      <c r="AD34" s="87" t="s">
+        <v>53</v>
+      </c>
+      <c r="AE34" s="88"/>
+      <c r="AF34" s="89"/>
+      <c r="AG34" s="87" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH34" s="88"/>
+      <c r="AI34" s="89"/>
+      <c r="AJ34" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="AK34" s="88"/>
+      <c r="AL34" s="89"/>
       <c r="AM34" s="84"/>
       <c r="AN34" s="73"/>
       <c r="AO34" s="71"/>
@@ -4115,51 +4142,44 @@
       <c r="BG34" s="71"/>
       <c r="BH34" s="72"/>
     </row>
-    <row r="35" spans="2:60">
-      <c r="B35" s="107" t="s">
-        <v>27</v>
-      </c>
-      <c r="C35" s="108"/>
-      <c r="D35" s="108"/>
-      <c r="E35" s="146">
-        <f>D7</f>
-        <v>0</v>
-      </c>
-      <c r="F35" s="146"/>
-      <c r="G35" s="146"/>
-      <c r="H35" s="146"/>
-      <c r="I35" s="146"/>
-      <c r="J35" s="146"/>
-      <c r="K35" s="146"/>
-      <c r="L35" s="146"/>
-      <c r="M35" s="146"/>
-      <c r="N35" s="146"/>
-      <c r="O35" s="146"/>
-      <c r="P35" s="146"/>
-      <c r="Q35" s="146"/>
-      <c r="R35" s="146"/>
-      <c r="S35" s="146"/>
-      <c r="T35" s="146"/>
-      <c r="U35" s="147"/>
-      <c r="V35" s="87" t="s">
-        <v>19</v>
-      </c>
-      <c r="W35" s="88"/>
-      <c r="X35" s="88"/>
-      <c r="Y35" s="88"/>
-      <c r="Z35" s="88"/>
-      <c r="AA35" s="88"/>
-      <c r="AB35" s="88"/>
-      <c r="AC35" s="88"/>
-      <c r="AD35" s="88"/>
-      <c r="AE35" s="88"/>
-      <c r="AF35" s="88"/>
-      <c r="AG35" s="88"/>
-      <c r="AH35" s="88"/>
-      <c r="AI35" s="88"/>
-      <c r="AJ35" s="88"/>
-      <c r="AK35" s="88"/>
-      <c r="AL35" s="89"/>
+    <row r="35" spans="2:60" ht="14.85" customHeight="1">
+      <c r="B35" s="36"/>
+      <c r="C35" s="110"/>
+      <c r="D35" s="148"/>
+      <c r="E35" s="149"/>
+      <c r="F35" s="149"/>
+      <c r="G35" s="149"/>
+      <c r="H35" s="149"/>
+      <c r="I35" s="149"/>
+      <c r="J35" s="149"/>
+      <c r="K35" s="149"/>
+      <c r="L35" s="149"/>
+      <c r="M35" s="149"/>
+      <c r="N35" s="149"/>
+      <c r="O35" s="149"/>
+      <c r="P35" s="149"/>
+      <c r="Q35" s="150"/>
+      <c r="R35" s="98"/>
+      <c r="S35" s="100"/>
+      <c r="T35" s="98"/>
+      <c r="U35" s="100"/>
+      <c r="V35" s="90"/>
+      <c r="W35" s="92"/>
+      <c r="X35" s="90"/>
+      <c r="Y35" s="91"/>
+      <c r="Z35" s="92"/>
+      <c r="AA35" s="90"/>
+      <c r="AB35" s="91"/>
+      <c r="AC35" s="92"/>
+      <c r="AD35" s="90"/>
+      <c r="AE35" s="91"/>
+      <c r="AF35" s="92"/>
+      <c r="AG35" s="90"/>
+      <c r="AH35" s="91"/>
+      <c r="AI35" s="92"/>
+      <c r="AJ35" s="90"/>
+      <c r="AK35" s="91"/>
+      <c r="AL35" s="92"/>
       <c r="AM35" s="84"/>
       <c r="AN35" s="73"/>
       <c r="AO35" s="71"/>
@@ -4187,64 +4207,44 @@
       <c r="BG35" s="71"/>
       <c r="BH35" s="72"/>
     </row>
-    <row r="36" spans="2:60">
-      <c r="B36" s="87" t="s">
-        <v>21</v>
-      </c>
-      <c r="C36" s="89"/>
-      <c r="D36" s="87" t="s">
-        <v>22</v>
-      </c>
-      <c r="E36" s="88"/>
-      <c r="F36" s="88"/>
-      <c r="G36" s="88"/>
-      <c r="H36" s="88"/>
-      <c r="I36" s="88"/>
-      <c r="J36" s="88"/>
-      <c r="K36" s="88"/>
-      <c r="L36" s="88"/>
-      <c r="M36" s="88"/>
-      <c r="N36" s="88"/>
-      <c r="O36" s="88"/>
-      <c r="P36" s="88"/>
-      <c r="Q36" s="89"/>
-      <c r="R36" s="87" t="s">
-        <v>14</v>
-      </c>
-      <c r="S36" s="89"/>
-      <c r="T36" s="87" t="s">
-        <v>15</v>
-      </c>
-      <c r="U36" s="89"/>
-      <c r="V36" s="87" t="s">
-        <v>16</v>
-      </c>
-      <c r="W36" s="89"/>
-      <c r="X36" s="87" t="s">
-        <v>53</v>
-      </c>
-      <c r="Y36" s="88"/>
-      <c r="Z36" s="89"/>
-      <c r="AA36" s="87" t="s">
-        <v>53</v>
-      </c>
-      <c r="AB36" s="88"/>
-      <c r="AC36" s="89"/>
-      <c r="AD36" s="87" t="s">
-        <v>53</v>
-      </c>
-      <c r="AE36" s="88"/>
-      <c r="AF36" s="89"/>
-      <c r="AG36" s="87" t="s">
-        <v>17</v>
-      </c>
-      <c r="AH36" s="88"/>
-      <c r="AI36" s="89"/>
-      <c r="AJ36" s="87" t="s">
-        <v>18</v>
-      </c>
-      <c r="AK36" s="88"/>
-      <c r="AL36" s="89"/>
+    <row r="36" spans="2:60" ht="14.85" customHeight="1">
+      <c r="B36" s="36"/>
+      <c r="C36" s="110"/>
+      <c r="D36" s="148"/>
+      <c r="E36" s="149"/>
+      <c r="F36" s="149"/>
+      <c r="G36" s="149"/>
+      <c r="H36" s="149"/>
+      <c r="I36" s="149"/>
+      <c r="J36" s="149"/>
+      <c r="K36" s="149"/>
+      <c r="L36" s="149"/>
+      <c r="M36" s="149"/>
+      <c r="N36" s="149"/>
+      <c r="O36" s="149"/>
+      <c r="P36" s="149"/>
+      <c r="Q36" s="150"/>
+      <c r="R36" s="98"/>
+      <c r="S36" s="100"/>
+      <c r="T36" s="98"/>
+      <c r="U36" s="100"/>
+      <c r="V36" s="90"/>
+      <c r="W36" s="92"/>
+      <c r="X36" s="90"/>
+      <c r="Y36" s="91"/>
+      <c r="Z36" s="92"/>
+      <c r="AA36" s="90"/>
+      <c r="AB36" s="91"/>
+      <c r="AC36" s="92"/>
+      <c r="AD36" s="90"/>
+      <c r="AE36" s="91"/>
+      <c r="AF36" s="92"/>
+      <c r="AG36" s="90"/>
+      <c r="AH36" s="91"/>
+      <c r="AI36" s="92"/>
+      <c r="AJ36" s="90"/>
+      <c r="AK36" s="91"/>
+      <c r="AL36" s="92"/>
       <c r="AM36" s="84"/>
       <c r="AN36" s="73"/>
       <c r="AO36" s="71"/>
@@ -4272,7 +4272,7 @@
       <c r="BG36" s="71"/>
       <c r="BH36" s="72"/>
     </row>
-    <row r="37" spans="2:60">
+    <row r="37" spans="2:60" ht="14.85" customHeight="1">
       <c r="B37" s="36"/>
       <c r="C37" s="110"/>
       <c r="D37" s="148"/>
@@ -4337,7 +4337,7 @@
       <c r="BG37" s="71"/>
       <c r="BH37" s="72"/>
     </row>
-    <row r="38" spans="2:60">
+    <row r="38" spans="2:60" ht="14.85" customHeight="1">
       <c r="B38" s="36"/>
       <c r="C38" s="110"/>
       <c r="D38" s="148"/>
@@ -4402,7 +4402,7 @@
       <c r="BG38" s="71"/>
       <c r="BH38" s="72"/>
     </row>
-    <row r="39" spans="2:60">
+    <row r="39" spans="2:60" ht="14.85" customHeight="1">
       <c r="B39" s="36"/>
       <c r="C39" s="110"/>
       <c r="D39" s="148"/>
@@ -4467,7 +4467,7 @@
       <c r="BG39" s="71"/>
       <c r="BH39" s="72"/>
     </row>
-    <row r="40" spans="2:60">
+    <row r="40" spans="2:60" ht="14.85" customHeight="1">
       <c r="B40" s="36"/>
       <c r="C40" s="110"/>
       <c r="D40" s="148"/>
@@ -4532,7 +4532,7 @@
       <c r="BG40" s="71"/>
       <c r="BH40" s="72"/>
     </row>
-    <row r="41" spans="2:60">
+    <row r="41" spans="2:60" ht="14.85" customHeight="1">
       <c r="B41" s="36"/>
       <c r="C41" s="110"/>
       <c r="D41" s="148"/>
@@ -4597,7 +4597,7 @@
       <c r="BG41" s="71"/>
       <c r="BH41" s="72"/>
     </row>
-    <row r="42" spans="2:60">
+    <row r="42" spans="2:60" ht="14.85" customHeight="1">
       <c r="B42" s="36"/>
       <c r="C42" s="110"/>
       <c r="D42" s="148"/>
@@ -4662,7 +4662,7 @@
       <c r="BG42" s="71"/>
       <c r="BH42" s="72"/>
     </row>
-    <row r="43" spans="2:60">
+    <row r="43" spans="2:60" ht="14.85" customHeight="1">
       <c r="B43" s="36"/>
       <c r="C43" s="110"/>
       <c r="D43" s="148"/>
@@ -4727,7 +4727,7 @@
       <c r="BG43" s="71"/>
       <c r="BH43" s="72"/>
     </row>
-    <row r="44" spans="2:60">
+    <row r="44" spans="2:60" ht="14.85" customHeight="1">
       <c r="B44" s="36"/>
       <c r="C44" s="110"/>
       <c r="D44" s="148"/>
@@ -4792,7 +4792,7 @@
       <c r="BG44" s="71"/>
       <c r="BH44" s="72"/>
     </row>
-    <row r="45" spans="2:60">
+    <row r="45" spans="2:60" ht="14.85" customHeight="1">
       <c r="B45" s="36"/>
       <c r="C45" s="110"/>
       <c r="D45" s="148"/>
@@ -4857,7 +4857,7 @@
       <c r="BG45" s="71"/>
       <c r="BH45" s="72"/>
     </row>
-    <row r="46" spans="2:60">
+    <row r="46" spans="2:60" ht="14.85" customHeight="1">
       <c r="B46" s="36"/>
       <c r="C46" s="110"/>
       <c r="D46" s="148"/>
@@ -4922,7 +4922,7 @@
       <c r="BG46" s="71"/>
       <c r="BH46" s="72"/>
     </row>
-    <row r="47" spans="2:60">
+    <row r="47" spans="2:60" ht="14.85" customHeight="1">
       <c r="B47" s="36"/>
       <c r="C47" s="110"/>
       <c r="D47" s="148"/>
@@ -4987,7 +4987,7 @@
       <c r="BG47" s="71"/>
       <c r="BH47" s="72"/>
     </row>
-    <row r="48" spans="2:60">
+    <row r="48" spans="2:60" ht="14.85" customHeight="1">
       <c r="B48" s="36"/>
       <c r="C48" s="110"/>
       <c r="D48" s="148"/>
@@ -5052,7 +5052,7 @@
       <c r="BG48" s="71"/>
       <c r="BH48" s="72"/>
     </row>
-    <row r="49" spans="2:60">
+    <row r="49" spans="2:60" ht="14.85" customHeight="1">
       <c r="B49" s="36"/>
       <c r="C49" s="110"/>
       <c r="D49" s="148"/>
@@ -5117,7 +5117,7 @@
       <c r="BG49" s="71"/>
       <c r="BH49" s="72"/>
     </row>
-    <row r="50" spans="2:60">
+    <row r="50" spans="2:60" ht="14.85" customHeight="1">
       <c r="B50" s="36"/>
       <c r="C50" s="110"/>
       <c r="D50" s="148"/>
@@ -5182,44 +5182,54 @@
       <c r="BG50" s="71"/>
       <c r="BH50" s="72"/>
     </row>
-    <row r="51" spans="2:60">
-      <c r="B51" s="36"/>
-      <c r="C51" s="110"/>
-      <c r="D51" s="148"/>
-      <c r="E51" s="149"/>
-      <c r="F51" s="149"/>
-      <c r="G51" s="149"/>
-      <c r="H51" s="149"/>
-      <c r="I51" s="149"/>
-      <c r="J51" s="149"/>
-      <c r="K51" s="149"/>
-      <c r="L51" s="149"/>
-      <c r="M51" s="149"/>
-      <c r="N51" s="149"/>
-      <c r="O51" s="149"/>
-      <c r="P51" s="149"/>
-      <c r="Q51" s="150"/>
-      <c r="R51" s="98"/>
-      <c r="S51" s="100"/>
-      <c r="T51" s="98"/>
-      <c r="U51" s="100"/>
-      <c r="V51" s="90"/>
-      <c r="W51" s="92"/>
-      <c r="X51" s="90"/>
-      <c r="Y51" s="91"/>
-      <c r="Z51" s="92"/>
-      <c r="AA51" s="90"/>
-      <c r="AB51" s="91"/>
-      <c r="AC51" s="92"/>
-      <c r="AD51" s="90"/>
-      <c r="AE51" s="91"/>
-      <c r="AF51" s="92"/>
-      <c r="AG51" s="90"/>
-      <c r="AH51" s="91"/>
-      <c r="AI51" s="92"/>
-      <c r="AJ51" s="90"/>
-      <c r="AK51" s="91"/>
-      <c r="AL51" s="92"/>
+    <row r="51" spans="2:60" ht="13.95" customHeight="1">
+      <c r="B51" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C51" s="158"/>
+      <c r="D51" s="158"/>
+      <c r="E51" s="158"/>
+      <c r="F51" s="158"/>
+      <c r="G51" s="159"/>
+      <c r="H51" s="159"/>
+      <c r="I51" s="159"/>
+      <c r="J51" s="160"/>
+      <c r="K51" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="L51" s="129"/>
+      <c r="M51" s="129"/>
+      <c r="N51" s="129"/>
+      <c r="O51" s="129"/>
+      <c r="P51" s="129"/>
+      <c r="Q51" s="130"/>
+      <c r="R51" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="S51" s="129"/>
+      <c r="T51" s="129"/>
+      <c r="U51" s="129"/>
+      <c r="V51" s="129"/>
+      <c r="W51" s="129"/>
+      <c r="X51" s="130"/>
+      <c r="Y51" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z51" s="129"/>
+      <c r="AA51" s="129"/>
+      <c r="AB51" s="129"/>
+      <c r="AC51" s="129"/>
+      <c r="AD51" s="129"/>
+      <c r="AE51" s="130"/>
+      <c r="AF51" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AG51" s="129"/>
+      <c r="AH51" s="129"/>
+      <c r="AI51" s="129"/>
+      <c r="AJ51" s="129"/>
+      <c r="AK51" s="129"/>
+      <c r="AL51" s="130"/>
       <c r="AM51" s="84"/>
       <c r="AN51" s="73"/>
       <c r="AO51" s="71"/>
@@ -5247,174 +5257,170 @@
       <c r="BG51" s="71"/>
       <c r="BH51" s="72"/>
     </row>
-    <row r="52" spans="2:60">
-      <c r="B52" s="36"/>
-      <c r="C52" s="110"/>
-      <c r="D52" s="148"/>
-      <c r="E52" s="149"/>
-      <c r="F52" s="149"/>
-      <c r="G52" s="149"/>
-      <c r="H52" s="149"/>
-      <c r="I52" s="149"/>
-      <c r="J52" s="149"/>
-      <c r="K52" s="149"/>
-      <c r="L52" s="149"/>
-      <c r="M52" s="149"/>
-      <c r="N52" s="149"/>
-      <c r="O52" s="149"/>
-      <c r="P52" s="149"/>
-      <c r="Q52" s="150"/>
-      <c r="R52" s="98"/>
-      <c r="S52" s="100"/>
-      <c r="T52" s="98"/>
-      <c r="U52" s="100"/>
-      <c r="V52" s="90"/>
-      <c r="W52" s="92"/>
-      <c r="X52" s="90"/>
-      <c r="Y52" s="91"/>
-      <c r="Z52" s="92"/>
-      <c r="AA52" s="90"/>
-      <c r="AB52" s="91"/>
-      <c r="AC52" s="92"/>
-      <c r="AD52" s="90"/>
-      <c r="AE52" s="91"/>
-      <c r="AF52" s="92"/>
-      <c r="AG52" s="90"/>
-      <c r="AH52" s="91"/>
-      <c r="AI52" s="92"/>
-      <c r="AJ52" s="90"/>
-      <c r="AK52" s="91"/>
-      <c r="AL52" s="92"/>
-      <c r="AM52" s="84"/>
-      <c r="AN52" s="73"/>
-      <c r="AO52" s="71"/>
-      <c r="AP52" s="72"/>
-      <c r="AQ52" s="26"/>
-      <c r="AR52" s="27"/>
-      <c r="AS52" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT52" s="85"/>
-      <c r="AU52" s="86"/>
-      <c r="AV52" s="71"/>
-      <c r="AW52" s="72"/>
-      <c r="AX52" s="84"/>
-      <c r="AY52" s="73"/>
-      <c r="AZ52" s="71"/>
-      <c r="BA52" s="72"/>
-      <c r="BB52" s="26"/>
-      <c r="BC52" s="27"/>
-      <c r="BD52" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE52" s="85"/>
-      <c r="BF52" s="86"/>
-      <c r="BG52" s="71"/>
-      <c r="BH52" s="72"/>
+    <row r="52" spans="2:60" ht="6.6" customHeight="1">
+      <c r="B52" s="151"/>
+      <c r="C52" s="152"/>
+      <c r="D52" s="152"/>
+      <c r="E52" s="152"/>
+      <c r="F52" s="152"/>
+      <c r="G52" s="161"/>
+      <c r="H52" s="161"/>
+      <c r="I52" s="161"/>
+      <c r="J52" s="162"/>
+      <c r="K52" s="175"/>
+      <c r="L52" s="176"/>
+      <c r="M52" s="176"/>
+      <c r="N52" s="176"/>
+      <c r="O52" s="176"/>
+      <c r="P52" s="176"/>
+      <c r="Q52" s="177"/>
+      <c r="R52" s="175"/>
+      <c r="S52" s="176"/>
+      <c r="T52" s="176"/>
+      <c r="U52" s="176"/>
+      <c r="V52" s="176"/>
+      <c r="W52" s="176"/>
+      <c r="X52" s="177"/>
+      <c r="Y52" s="175"/>
+      <c r="Z52" s="176"/>
+      <c r="AA52" s="176"/>
+      <c r="AB52" s="176"/>
+      <c r="AC52" s="176"/>
+      <c r="AD52" s="176"/>
+      <c r="AE52" s="177"/>
+      <c r="AF52" s="175"/>
+      <c r="AG52" s="176"/>
+      <c r="AH52" s="176"/>
+      <c r="AI52" s="176"/>
+      <c r="AJ52" s="176"/>
+      <c r="AK52" s="176"/>
+      <c r="AL52" s="177"/>
+      <c r="AM52" s="187"/>
+      <c r="AN52" s="188"/>
+      <c r="AO52" s="191"/>
+      <c r="AP52" s="192"/>
+      <c r="AQ52" s="191"/>
+      <c r="AR52" s="195"/>
+      <c r="AS52" s="197" t="s">
+        <v>5</v>
+      </c>
+      <c r="AT52" s="199"/>
+      <c r="AU52" s="200"/>
+      <c r="AV52" s="203"/>
+      <c r="AW52" s="200"/>
+      <c r="AX52" s="205"/>
+      <c r="AY52" s="206"/>
+      <c r="AZ52" s="203"/>
+      <c r="BA52" s="200"/>
+      <c r="BB52" s="203"/>
+      <c r="BC52" s="199"/>
+      <c r="BD52" s="197" t="s">
+        <v>5</v>
+      </c>
+      <c r="BE52" s="199"/>
+      <c r="BF52" s="200"/>
+      <c r="BG52" s="203"/>
+      <c r="BH52" s="200"/>
     </row>
-    <row r="53" spans="2:60">
-      <c r="B53" s="36"/>
-      <c r="C53" s="110"/>
-      <c r="D53" s="148"/>
-      <c r="E53" s="149"/>
-      <c r="F53" s="149"/>
-      <c r="G53" s="149"/>
-      <c r="H53" s="149"/>
-      <c r="I53" s="149"/>
-      <c r="J53" s="149"/>
-      <c r="K53" s="149"/>
-      <c r="L53" s="149"/>
-      <c r="M53" s="149"/>
-      <c r="N53" s="149"/>
-      <c r="O53" s="149"/>
-      <c r="P53" s="149"/>
-      <c r="Q53" s="150"/>
-      <c r="R53" s="98"/>
-      <c r="S53" s="100"/>
-      <c r="T53" s="98"/>
-      <c r="U53" s="100"/>
-      <c r="V53" s="90"/>
-      <c r="W53" s="92"/>
-      <c r="X53" s="90"/>
-      <c r="Y53" s="91"/>
-      <c r="Z53" s="92"/>
-      <c r="AA53" s="90"/>
-      <c r="AB53" s="91"/>
-      <c r="AC53" s="92"/>
-      <c r="AD53" s="90"/>
-      <c r="AE53" s="91"/>
-      <c r="AF53" s="92"/>
-      <c r="AG53" s="90"/>
-      <c r="AH53" s="91"/>
-      <c r="AI53" s="92"/>
-      <c r="AJ53" s="90"/>
-      <c r="AK53" s="91"/>
-      <c r="AL53" s="92"/>
-      <c r="AM53" s="84"/>
-      <c r="AN53" s="73"/>
-      <c r="AO53" s="71"/>
-      <c r="AP53" s="72"/>
-      <c r="AQ53" s="26"/>
-      <c r="AR53" s="27"/>
-      <c r="AS53" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT53" s="85"/>
-      <c r="AU53" s="86"/>
-      <c r="AV53" s="71"/>
-      <c r="AW53" s="72"/>
-      <c r="AX53" s="84"/>
-      <c r="AY53" s="73"/>
-      <c r="AZ53" s="71"/>
-      <c r="BA53" s="72"/>
-      <c r="BB53" s="26"/>
-      <c r="BC53" s="27"/>
-      <c r="BD53" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE53" s="85"/>
-      <c r="BF53" s="86"/>
-      <c r="BG53" s="71"/>
-      <c r="BH53" s="72"/>
+    <row r="53" spans="2:60" ht="6.6" customHeight="1">
+      <c r="B53" s="153"/>
+      <c r="C53" s="154"/>
+      <c r="D53" s="154"/>
+      <c r="E53" s="154"/>
+      <c r="F53" s="154"/>
+      <c r="G53" s="161"/>
+      <c r="H53" s="161"/>
+      <c r="I53" s="161"/>
+      <c r="J53" s="162"/>
+      <c r="K53" s="126"/>
+      <c r="L53" s="127"/>
+      <c r="M53" s="127"/>
+      <c r="N53" s="127"/>
+      <c r="O53" s="127"/>
+      <c r="P53" s="127"/>
+      <c r="Q53" s="128"/>
+      <c r="R53" s="126"/>
+      <c r="S53" s="127"/>
+      <c r="T53" s="127"/>
+      <c r="U53" s="127"/>
+      <c r="V53" s="127"/>
+      <c r="W53" s="127"/>
+      <c r="X53" s="128"/>
+      <c r="Y53" s="126"/>
+      <c r="Z53" s="127"/>
+      <c r="AA53" s="127"/>
+      <c r="AB53" s="127"/>
+      <c r="AC53" s="127"/>
+      <c r="AD53" s="127"/>
+      <c r="AE53" s="128"/>
+      <c r="AF53" s="126"/>
+      <c r="AG53" s="127"/>
+      <c r="AH53" s="127"/>
+      <c r="AI53" s="127"/>
+      <c r="AJ53" s="127"/>
+      <c r="AK53" s="127"/>
+      <c r="AL53" s="128"/>
+      <c r="AM53" s="189"/>
+      <c r="AN53" s="190"/>
+      <c r="AO53" s="193"/>
+      <c r="AP53" s="194"/>
+      <c r="AQ53" s="193"/>
+      <c r="AR53" s="196"/>
+      <c r="AS53" s="198"/>
+      <c r="AT53" s="201"/>
+      <c r="AU53" s="202"/>
+      <c r="AV53" s="204"/>
+      <c r="AW53" s="202"/>
+      <c r="AX53" s="207"/>
+      <c r="AY53" s="208"/>
+      <c r="AZ53" s="204"/>
+      <c r="BA53" s="202"/>
+      <c r="BB53" s="204"/>
+      <c r="BC53" s="201"/>
+      <c r="BD53" s="198"/>
+      <c r="BE53" s="201"/>
+      <c r="BF53" s="202"/>
+      <c r="BG53" s="204"/>
+      <c r="BH53" s="202"/>
     </row>
     <row r="54" spans="2:60">
-      <c r="B54" s="36"/>
-      <c r="C54" s="110"/>
-      <c r="D54" s="148"/>
-      <c r="E54" s="149"/>
-      <c r="F54" s="149"/>
-      <c r="G54" s="149"/>
-      <c r="H54" s="149"/>
-      <c r="I54" s="149"/>
-      <c r="J54" s="149"/>
-      <c r="K54" s="149"/>
-      <c r="L54" s="149"/>
-      <c r="M54" s="149"/>
-      <c r="N54" s="149"/>
-      <c r="O54" s="149"/>
-      <c r="P54" s="149"/>
-      <c r="Q54" s="150"/>
-      <c r="R54" s="98"/>
-      <c r="S54" s="100"/>
-      <c r="T54" s="98"/>
-      <c r="U54" s="100"/>
-      <c r="V54" s="90"/>
-      <c r="W54" s="92"/>
-      <c r="X54" s="90"/>
-      <c r="Y54" s="91"/>
-      <c r="Z54" s="92"/>
-      <c r="AA54" s="90"/>
-      <c r="AB54" s="91"/>
-      <c r="AC54" s="92"/>
-      <c r="AD54" s="90"/>
-      <c r="AE54" s="91"/>
-      <c r="AF54" s="92"/>
-      <c r="AG54" s="90"/>
-      <c r="AH54" s="91"/>
-      <c r="AI54" s="92"/>
-      <c r="AJ54" s="90"/>
-      <c r="AK54" s="91"/>
-      <c r="AL54" s="92"/>
+      <c r="B54" s="163"/>
+      <c r="C54" s="164"/>
+      <c r="D54" s="164"/>
+      <c r="E54" s="164"/>
+      <c r="F54" s="164"/>
+      <c r="G54" s="164"/>
+      <c r="H54" s="164"/>
+      <c r="I54" s="164"/>
+      <c r="J54" s="165"/>
+      <c r="K54" s="157"/>
+      <c r="L54" s="155"/>
+      <c r="M54" s="155"/>
+      <c r="N54" s="155"/>
+      <c r="O54" s="155"/>
+      <c r="P54" s="155"/>
+      <c r="Q54" s="156"/>
+      <c r="R54" s="157"/>
+      <c r="S54" s="155"/>
+      <c r="T54" s="155"/>
+      <c r="U54" s="155"/>
+      <c r="V54" s="155"/>
+      <c r="W54" s="155"/>
+      <c r="X54" s="156"/>
+      <c r="Y54" s="157"/>
+      <c r="Z54" s="155"/>
+      <c r="AA54" s="155"/>
+      <c r="AB54" s="155"/>
+      <c r="AC54" s="155"/>
+      <c r="AD54" s="155"/>
+      <c r="AE54" s="156"/>
+      <c r="AF54" s="157"/>
+      <c r="AG54" s="155"/>
+      <c r="AH54" s="155"/>
+      <c r="AI54" s="155"/>
+      <c r="AJ54" s="155"/>
+      <c r="AK54" s="155"/>
+      <c r="AL54" s="156"/>
       <c r="AM54" s="84"/>
       <c r="AN54" s="73"/>
       <c r="AO54" s="71"/>
@@ -5442,54 +5448,54 @@
       <c r="BG54" s="71"/>
       <c r="BH54" s="72"/>
     </row>
-    <row r="55" spans="2:60" ht="13.95" customHeight="1">
-      <c r="B55" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C55" s="158"/>
-      <c r="D55" s="158"/>
-      <c r="E55" s="158"/>
-      <c r="F55" s="158"/>
-      <c r="G55" s="159"/>
-      <c r="H55" s="159"/>
-      <c r="I55" s="159"/>
-      <c r="J55" s="160"/>
-      <c r="K55" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="L55" s="129"/>
-      <c r="M55" s="129"/>
-      <c r="N55" s="129"/>
-      <c r="O55" s="129"/>
-      <c r="P55" s="129"/>
-      <c r="Q55" s="130"/>
-      <c r="R55" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="S55" s="129"/>
-      <c r="T55" s="129"/>
-      <c r="U55" s="129"/>
-      <c r="V55" s="129"/>
-      <c r="W55" s="129"/>
-      <c r="X55" s="130"/>
-      <c r="Y55" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="Z55" s="129"/>
-      <c r="AA55" s="129"/>
-      <c r="AB55" s="129"/>
-      <c r="AC55" s="129"/>
-      <c r="AD55" s="129"/>
-      <c r="AE55" s="130"/>
-      <c r="AF55" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="AG55" s="129"/>
-      <c r="AH55" s="129"/>
-      <c r="AI55" s="129"/>
-      <c r="AJ55" s="129"/>
-      <c r="AK55" s="129"/>
-      <c r="AL55" s="130"/>
+    <row r="55" spans="2:60">
+      <c r="B55" s="166" t="s">
+        <v>25</v>
+      </c>
+      <c r="C55" s="167"/>
+      <c r="D55" s="167"/>
+      <c r="E55" s="167"/>
+      <c r="F55" s="167"/>
+      <c r="G55" s="167"/>
+      <c r="H55" s="167"/>
+      <c r="I55" s="167"/>
+      <c r="J55" s="168"/>
+      <c r="K55" s="166" t="s">
+        <v>26</v>
+      </c>
+      <c r="L55" s="167"/>
+      <c r="M55" s="167"/>
+      <c r="N55" s="167"/>
+      <c r="O55" s="167"/>
+      <c r="P55" s="167"/>
+      <c r="Q55" s="168"/>
+      <c r="R55" s="166" t="s">
+        <v>26</v>
+      </c>
+      <c r="S55" s="167"/>
+      <c r="T55" s="167"/>
+      <c r="U55" s="167"/>
+      <c r="V55" s="167"/>
+      <c r="W55" s="167"/>
+      <c r="X55" s="168"/>
+      <c r="Y55" s="166" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z55" s="167"/>
+      <c r="AA55" s="167"/>
+      <c r="AB55" s="167"/>
+      <c r="AC55" s="167"/>
+      <c r="AD55" s="167"/>
+      <c r="AE55" s="168"/>
+      <c r="AF55" s="166" t="s">
+        <v>26</v>
+      </c>
+      <c r="AG55" s="167"/>
+      <c r="AH55" s="167"/>
+      <c r="AI55" s="167"/>
+      <c r="AJ55" s="167"/>
+      <c r="AK55" s="167"/>
+      <c r="AL55" s="168"/>
       <c r="AM55" s="84"/>
       <c r="AN55" s="73"/>
       <c r="AO55" s="71"/>
@@ -5517,170 +5523,184 @@
       <c r="BG55" s="71"/>
       <c r="BH55" s="72"/>
     </row>
-    <row r="56" spans="2:60" ht="6.6" customHeight="1">
-      <c r="B56" s="151"/>
-      <c r="C56" s="152"/>
-      <c r="D56" s="152"/>
-      <c r="E56" s="152"/>
-      <c r="F56" s="152"/>
-      <c r="G56" s="161"/>
-      <c r="H56" s="161"/>
-      <c r="I56" s="161"/>
-      <c r="J56" s="162"/>
-      <c r="K56" s="175"/>
-      <c r="L56" s="176"/>
-      <c r="M56" s="176"/>
-      <c r="N56" s="176"/>
-      <c r="O56" s="176"/>
-      <c r="P56" s="176"/>
-      <c r="Q56" s="177"/>
-      <c r="R56" s="175"/>
-      <c r="S56" s="176"/>
-      <c r="T56" s="176"/>
-      <c r="U56" s="176"/>
-      <c r="V56" s="176"/>
-      <c r="W56" s="176"/>
-      <c r="X56" s="177"/>
-      <c r="Y56" s="175"/>
-      <c r="Z56" s="176"/>
-      <c r="AA56" s="176"/>
-      <c r="AB56" s="176"/>
-      <c r="AC56" s="176"/>
-      <c r="AD56" s="176"/>
-      <c r="AE56" s="177"/>
-      <c r="AF56" s="175"/>
-      <c r="AG56" s="176"/>
-      <c r="AH56" s="176"/>
-      <c r="AI56" s="176"/>
-      <c r="AJ56" s="176"/>
-      <c r="AK56" s="176"/>
-      <c r="AL56" s="177"/>
-      <c r="AM56" s="187"/>
-      <c r="AN56" s="188"/>
-      <c r="AO56" s="191"/>
-      <c r="AP56" s="192"/>
-      <c r="AQ56" s="191"/>
-      <c r="AR56" s="195"/>
-      <c r="AS56" s="197" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT56" s="199"/>
-      <c r="AU56" s="200"/>
-      <c r="AV56" s="203"/>
-      <c r="AW56" s="200"/>
-      <c r="AX56" s="205"/>
-      <c r="AY56" s="206"/>
-      <c r="AZ56" s="203"/>
-      <c r="BA56" s="200"/>
-      <c r="BB56" s="203"/>
-      <c r="BC56" s="199"/>
-      <c r="BD56" s="197" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE56" s="199"/>
-      <c r="BF56" s="200"/>
-      <c r="BG56" s="203"/>
-      <c r="BH56" s="200"/>
+    <row r="56" spans="2:60">
+      <c r="B56" s="169"/>
+      <c r="C56" s="170"/>
+      <c r="D56" s="170"/>
+      <c r="E56" s="170"/>
+      <c r="F56" s="170"/>
+      <c r="G56" s="170"/>
+      <c r="H56" s="170"/>
+      <c r="I56" s="170"/>
+      <c r="J56" s="171"/>
+      <c r="K56" s="169"/>
+      <c r="L56" s="170"/>
+      <c r="M56" s="170"/>
+      <c r="N56" s="170"/>
+      <c r="O56" s="170"/>
+      <c r="P56" s="170"/>
+      <c r="Q56" s="171"/>
+      <c r="R56" s="169"/>
+      <c r="S56" s="170"/>
+      <c r="T56" s="170"/>
+      <c r="U56" s="170"/>
+      <c r="V56" s="170"/>
+      <c r="W56" s="170"/>
+      <c r="X56" s="171"/>
+      <c r="Y56" s="169"/>
+      <c r="Z56" s="170"/>
+      <c r="AA56" s="170"/>
+      <c r="AB56" s="170"/>
+      <c r="AC56" s="170"/>
+      <c r="AD56" s="170"/>
+      <c r="AE56" s="171"/>
+      <c r="AF56" s="169"/>
+      <c r="AG56" s="170"/>
+      <c r="AH56" s="170"/>
+      <c r="AI56" s="170"/>
+      <c r="AJ56" s="170"/>
+      <c r="AK56" s="170"/>
+      <c r="AL56" s="171"/>
+      <c r="AM56" s="84"/>
+      <c r="AN56" s="73"/>
+      <c r="AO56" s="71"/>
+      <c r="AP56" s="72"/>
+      <c r="AQ56" s="26"/>
+      <c r="AR56" s="27"/>
+      <c r="AS56" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="AT56" s="85"/>
+      <c r="AU56" s="86"/>
+      <c r="AV56" s="71"/>
+      <c r="AW56" s="72"/>
+      <c r="AX56" s="84"/>
+      <c r="AY56" s="73"/>
+      <c r="AZ56" s="71"/>
+      <c r="BA56" s="72"/>
+      <c r="BB56" s="26"/>
+      <c r="BC56" s="27"/>
+      <c r="BD56" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="BE56" s="85"/>
+      <c r="BF56" s="86"/>
+      <c r="BG56" s="71"/>
+      <c r="BH56" s="72"/>
     </row>
-    <row r="57" spans="2:60" ht="6.6" customHeight="1">
-      <c r="B57" s="153"/>
-      <c r="C57" s="154"/>
-      <c r="D57" s="154"/>
-      <c r="E57" s="154"/>
-      <c r="F57" s="154"/>
-      <c r="G57" s="161"/>
-      <c r="H57" s="161"/>
-      <c r="I57" s="161"/>
-      <c r="J57" s="162"/>
-      <c r="K57" s="126"/>
-      <c r="L57" s="127"/>
-      <c r="M57" s="127"/>
-      <c r="N57" s="127"/>
-      <c r="O57" s="127"/>
-      <c r="P57" s="127"/>
-      <c r="Q57" s="128"/>
-      <c r="R57" s="126"/>
-      <c r="S57" s="127"/>
-      <c r="T57" s="127"/>
-      <c r="U57" s="127"/>
-      <c r="V57" s="127"/>
-      <c r="W57" s="127"/>
-      <c r="X57" s="128"/>
-      <c r="Y57" s="126"/>
-      <c r="Z57" s="127"/>
-      <c r="AA57" s="127"/>
-      <c r="AB57" s="127"/>
-      <c r="AC57" s="127"/>
-      <c r="AD57" s="127"/>
-      <c r="AE57" s="128"/>
-      <c r="AF57" s="126"/>
-      <c r="AG57" s="127"/>
-      <c r="AH57" s="127"/>
-      <c r="AI57" s="127"/>
-      <c r="AJ57" s="127"/>
-      <c r="AK57" s="127"/>
-      <c r="AL57" s="128"/>
-      <c r="AM57" s="189"/>
-      <c r="AN57" s="190"/>
-      <c r="AO57" s="193"/>
-      <c r="AP57" s="194"/>
-      <c r="AQ57" s="193"/>
-      <c r="AR57" s="196"/>
-      <c r="AS57" s="198"/>
-      <c r="AT57" s="201"/>
-      <c r="AU57" s="202"/>
-      <c r="AV57" s="204"/>
-      <c r="AW57" s="202"/>
-      <c r="AX57" s="207"/>
-      <c r="AY57" s="208"/>
-      <c r="AZ57" s="204"/>
-      <c r="BA57" s="202"/>
-      <c r="BB57" s="204"/>
-      <c r="BC57" s="201"/>
-      <c r="BD57" s="198"/>
-      <c r="BE57" s="201"/>
-      <c r="BF57" s="202"/>
-      <c r="BG57" s="204"/>
-      <c r="BH57" s="202"/>
+    <row r="57" spans="2:60">
+      <c r="B57" s="172" t="s">
+        <v>30</v>
+      </c>
+      <c r="C57" s="173"/>
+      <c r="D57" s="173"/>
+      <c r="E57" s="173"/>
+      <c r="F57" s="173"/>
+      <c r="G57" s="173"/>
+      <c r="H57" s="173"/>
+      <c r="I57" s="173"/>
+      <c r="J57" s="173"/>
+      <c r="K57" s="173"/>
+      <c r="L57" s="173"/>
+      <c r="M57" s="174"/>
+      <c r="N57" s="238" t="s">
+        <v>29</v>
+      </c>
+      <c r="O57" s="239"/>
+      <c r="P57" s="235"/>
+      <c r="Q57" s="235"/>
+      <c r="R57" s="244" t="s">
+        <v>28</v>
+      </c>
+      <c r="S57" s="245"/>
+      <c r="T57" s="236"/>
+      <c r="U57" s="236"/>
+      <c r="V57" s="81"/>
+      <c r="W57" s="82"/>
+      <c r="X57" s="82"/>
+      <c r="Y57" s="82"/>
+      <c r="Z57" s="82"/>
+      <c r="AA57" s="82"/>
+      <c r="AB57" s="82"/>
+      <c r="AC57" s="82"/>
+      <c r="AD57" s="82"/>
+      <c r="AE57" s="82"/>
+      <c r="AF57" s="82"/>
+      <c r="AG57" s="82"/>
+      <c r="AH57" s="82"/>
+      <c r="AI57" s="82"/>
+      <c r="AJ57" s="82"/>
+      <c r="AK57" s="82"/>
+      <c r="AL57" s="83"/>
+      <c r="AM57" s="84"/>
+      <c r="AN57" s="73"/>
+      <c r="AO57" s="71"/>
+      <c r="AP57" s="72"/>
+      <c r="AQ57" s="26"/>
+      <c r="AR57" s="27"/>
+      <c r="AS57" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="AT57" s="85"/>
+      <c r="AU57" s="86"/>
+      <c r="AV57" s="71"/>
+      <c r="AW57" s="72"/>
+      <c r="AX57" s="84"/>
+      <c r="AY57" s="73"/>
+      <c r="AZ57" s="71"/>
+      <c r="BA57" s="72"/>
+      <c r="BB57" s="26"/>
+      <c r="BC57" s="27"/>
+      <c r="BD57" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="BE57" s="85"/>
+      <c r="BF57" s="86"/>
+      <c r="BG57" s="71"/>
+      <c r="BH57" s="72"/>
     </row>
     <row r="58" spans="2:60">
-      <c r="B58" s="163"/>
-      <c r="C58" s="164"/>
-      <c r="D58" s="164"/>
-      <c r="E58" s="164"/>
-      <c r="F58" s="164"/>
-      <c r="G58" s="164"/>
-      <c r="H58" s="164"/>
-      <c r="I58" s="164"/>
-      <c r="J58" s="165"/>
-      <c r="K58" s="157"/>
-      <c r="L58" s="155"/>
-      <c r="M58" s="155"/>
-      <c r="N58" s="155"/>
-      <c r="O58" s="155"/>
-      <c r="P58" s="155"/>
-      <c r="Q58" s="156"/>
-      <c r="R58" s="157"/>
-      <c r="S58" s="155"/>
-      <c r="T58" s="155"/>
-      <c r="U58" s="155"/>
-      <c r="V58" s="155"/>
-      <c r="W58" s="155"/>
-      <c r="X58" s="156"/>
-      <c r="Y58" s="157"/>
-      <c r="Z58" s="155"/>
-      <c r="AA58" s="155"/>
-      <c r="AB58" s="155"/>
-      <c r="AC58" s="155"/>
-      <c r="AD58" s="155"/>
-      <c r="AE58" s="156"/>
-      <c r="AF58" s="157"/>
-      <c r="AG58" s="155"/>
-      <c r="AH58" s="155"/>
-      <c r="AI58" s="155"/>
-      <c r="AJ58" s="155"/>
-      <c r="AK58" s="155"/>
-      <c r="AL58" s="156"/>
+      <c r="B58" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="15"/>
+      <c r="H58" s="88"/>
+      <c r="I58" s="88"/>
+      <c r="J58" s="89"/>
+      <c r="K58" s="209" t="s">
+        <v>34</v>
+      </c>
+      <c r="L58" s="210"/>
+      <c r="M58" s="210"/>
+      <c r="N58" s="210"/>
+      <c r="O58" s="210"/>
+      <c r="P58" s="210"/>
+      <c r="Q58" s="210"/>
+      <c r="R58" s="246"/>
+      <c r="S58" s="246"/>
+      <c r="T58" s="246"/>
+      <c r="U58" s="247"/>
+      <c r="V58" s="61"/>
+      <c r="W58" s="59"/>
+      <c r="X58" s="59"/>
+      <c r="Y58" s="59"/>
+      <c r="Z58" s="59"/>
+      <c r="AA58" s="59"/>
+      <c r="AB58" s="59"/>
+      <c r="AC58" s="59"/>
+      <c r="AD58" s="59"/>
+      <c r="AE58" s="59"/>
+      <c r="AF58" s="59"/>
+      <c r="AG58" s="59"/>
+      <c r="AH58" s="59"/>
+      <c r="AI58" s="59"/>
+      <c r="AJ58" s="59"/>
+      <c r="AK58" s="59"/>
+      <c r="AL58" s="63"/>
       <c r="AM58" s="84"/>
       <c r="AN58" s="73"/>
       <c r="AO58" s="71"/>
@@ -5709,53 +5729,49 @@
       <c r="BH58" s="72"/>
     </row>
     <row r="59" spans="2:60">
-      <c r="B59" s="166" t="s">
-        <v>25</v>
-      </c>
-      <c r="C59" s="167"/>
-      <c r="D59" s="167"/>
-      <c r="E59" s="167"/>
-      <c r="F59" s="167"/>
-      <c r="G59" s="167"/>
-      <c r="H59" s="167"/>
-      <c r="I59" s="167"/>
-      <c r="J59" s="168"/>
-      <c r="K59" s="166" t="s">
-        <v>26</v>
-      </c>
-      <c r="L59" s="167"/>
-      <c r="M59" s="167"/>
-      <c r="N59" s="167"/>
-      <c r="O59" s="167"/>
-      <c r="P59" s="167"/>
-      <c r="Q59" s="168"/>
-      <c r="R59" s="166" t="s">
-        <v>26</v>
-      </c>
-      <c r="S59" s="167"/>
-      <c r="T59" s="167"/>
-      <c r="U59" s="167"/>
-      <c r="V59" s="167"/>
-      <c r="W59" s="167"/>
-      <c r="X59" s="168"/>
-      <c r="Y59" s="166" t="s">
-        <v>26</v>
-      </c>
-      <c r="Z59" s="167"/>
-      <c r="AA59" s="167"/>
-      <c r="AB59" s="167"/>
-      <c r="AC59" s="167"/>
-      <c r="AD59" s="167"/>
-      <c r="AE59" s="168"/>
-      <c r="AF59" s="166" t="s">
-        <v>26</v>
-      </c>
-      <c r="AG59" s="167"/>
-      <c r="AH59" s="167"/>
-      <c r="AI59" s="167"/>
-      <c r="AJ59" s="167"/>
-      <c r="AK59" s="167"/>
-      <c r="AL59" s="168"/>
+      <c r="B59" s="172" t="s">
+        <v>33</v>
+      </c>
+      <c r="C59" s="173"/>
+      <c r="D59" s="173"/>
+      <c r="E59" s="173"/>
+      <c r="F59" s="173"/>
+      <c r="G59" s="173"/>
+      <c r="H59" s="173"/>
+      <c r="I59" s="173"/>
+      <c r="J59" s="173"/>
+      <c r="K59" s="173"/>
+      <c r="L59" s="173"/>
+      <c r="M59" s="174"/>
+      <c r="N59" s="240" t="s">
+        <v>31</v>
+      </c>
+      <c r="O59" s="241"/>
+      <c r="P59" s="235"/>
+      <c r="Q59" s="235"/>
+      <c r="R59" s="242" t="s">
+        <v>32</v>
+      </c>
+      <c r="S59" s="243"/>
+      <c r="T59" s="237"/>
+      <c r="U59" s="237"/>
+      <c r="V59" s="61"/>
+      <c r="W59" s="258"/>
+      <c r="X59" s="258"/>
+      <c r="Y59" s="258"/>
+      <c r="Z59" s="258"/>
+      <c r="AA59" s="258"/>
+      <c r="AB59" s="258"/>
+      <c r="AC59" s="258"/>
+      <c r="AD59" s="258"/>
+      <c r="AE59" s="258"/>
+      <c r="AF59" s="59"/>
+      <c r="AG59" s="59"/>
+      <c r="AH59" s="59"/>
+      <c r="AI59" s="59"/>
+      <c r="AJ59" s="59"/>
+      <c r="AK59" s="59"/>
+      <c r="AL59" s="63"/>
       <c r="AM59" s="84"/>
       <c r="AN59" s="73"/>
       <c r="AO59" s="71"/>
@@ -5784,439 +5800,443 @@
       <c r="BH59" s="72"/>
     </row>
     <row r="60" spans="2:60">
-      <c r="B60" s="169"/>
-      <c r="C60" s="170"/>
-      <c r="D60" s="170"/>
-      <c r="E60" s="170"/>
-      <c r="F60" s="170"/>
-      <c r="G60" s="170"/>
-      <c r="H60" s="170"/>
-      <c r="I60" s="170"/>
-      <c r="J60" s="171"/>
-      <c r="K60" s="169"/>
-      <c r="L60" s="170"/>
-      <c r="M60" s="170"/>
-      <c r="N60" s="170"/>
-      <c r="O60" s="170"/>
-      <c r="P60" s="170"/>
-      <c r="Q60" s="171"/>
-      <c r="R60" s="169"/>
-      <c r="S60" s="170"/>
-      <c r="T60" s="170"/>
-      <c r="U60" s="170"/>
-      <c r="V60" s="170"/>
-      <c r="W60" s="170"/>
-      <c r="X60" s="171"/>
-      <c r="Y60" s="169"/>
-      <c r="Z60" s="170"/>
-      <c r="AA60" s="170"/>
-      <c r="AB60" s="170"/>
-      <c r="AC60" s="170"/>
-      <c r="AD60" s="170"/>
-      <c r="AE60" s="171"/>
-      <c r="AF60" s="169"/>
-      <c r="AG60" s="170"/>
-      <c r="AH60" s="170"/>
-      <c r="AI60" s="170"/>
-      <c r="AJ60" s="170"/>
-      <c r="AK60" s="170"/>
-      <c r="AL60" s="171"/>
-      <c r="AM60" s="84"/>
-      <c r="AN60" s="73"/>
-      <c r="AO60" s="71"/>
-      <c r="AP60" s="72"/>
-      <c r="AQ60" s="26"/>
-      <c r="AR60" s="27"/>
-      <c r="AS60" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT60" s="85"/>
-      <c r="AU60" s="86"/>
-      <c r="AV60" s="71"/>
-      <c r="AW60" s="72"/>
-      <c r="AX60" s="84"/>
-      <c r="AY60" s="73"/>
-      <c r="AZ60" s="71"/>
-      <c r="BA60" s="72"/>
-      <c r="BB60" s="26"/>
-      <c r="BC60" s="27"/>
-      <c r="BD60" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE60" s="85"/>
-      <c r="BF60" s="86"/>
-      <c r="BG60" s="71"/>
-      <c r="BH60" s="72"/>
+      <c r="B60" s="248" t="s">
+        <v>44</v>
+      </c>
+      <c r="C60" s="249"/>
+      <c r="D60" s="249"/>
+      <c r="E60" s="249"/>
+      <c r="F60" s="249"/>
+      <c r="G60" s="249"/>
+      <c r="H60" s="249"/>
+      <c r="I60" s="249"/>
+      <c r="J60" s="249"/>
+      <c r="K60" s="249"/>
+      <c r="L60" s="249"/>
+      <c r="M60" s="250"/>
+      <c r="N60" s="240" t="s">
+        <v>31</v>
+      </c>
+      <c r="O60" s="241"/>
+      <c r="P60" s="235"/>
+      <c r="Q60" s="235"/>
+      <c r="R60" s="240" t="s">
+        <v>32</v>
+      </c>
+      <c r="S60" s="241"/>
+      <c r="T60" s="235"/>
+      <c r="U60" s="235"/>
+      <c r="V60" s="62"/>
+      <c r="W60" s="60"/>
+      <c r="X60" s="60"/>
+      <c r="Y60" s="60"/>
+      <c r="Z60" s="60"/>
+      <c r="AA60" s="60"/>
+      <c r="AB60" s="60"/>
+      <c r="AC60" s="60"/>
+      <c r="AD60" s="60"/>
+      <c r="AE60" s="60"/>
+      <c r="AF60" s="60"/>
+      <c r="AG60" s="60"/>
+      <c r="AH60" s="60"/>
+      <c r="AI60" s="60"/>
+      <c r="AJ60" s="60"/>
+      <c r="AK60" s="60"/>
+      <c r="AL60" s="64"/>
+      <c r="AM60" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="AN60" s="25"/>
+      <c r="AO60" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="AP60" s="25"/>
+      <c r="AQ60" s="25"/>
+      <c r="AR60" s="25"/>
+      <c r="AS60" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="AT60" s="25"/>
+      <c r="AU60" s="25"/>
+      <c r="AV60" s="25"/>
+      <c r="AW60" s="25"/>
+      <c r="AX60" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="AY60" s="25"/>
+      <c r="AZ60" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="BA60" s="25"/>
+      <c r="BB60" s="25"/>
+      <c r="BC60" s="25"/>
+      <c r="BD60" s="25" t="s">
+        <v>47</v>
+      </c>
+      <c r="BE60" s="25"/>
+      <c r="BF60" s="25"/>
+      <c r="BG60" s="25"/>
+      <c r="BH60" s="25"/>
     </row>
-    <row r="61" spans="2:60">
-      <c r="B61" s="172" t="s">
-        <v>30</v>
-      </c>
-      <c r="C61" s="173"/>
-      <c r="D61" s="173"/>
-      <c r="E61" s="173"/>
-      <c r="F61" s="173"/>
-      <c r="G61" s="173"/>
-      <c r="H61" s="173"/>
-      <c r="I61" s="173"/>
-      <c r="J61" s="173"/>
-      <c r="K61" s="173"/>
-      <c r="L61" s="173"/>
-      <c r="M61" s="174"/>
-      <c r="N61" s="238" t="s">
-        <v>29</v>
-      </c>
-      <c r="O61" s="239"/>
-      <c r="P61" s="235"/>
-      <c r="Q61" s="235"/>
-      <c r="R61" s="244" t="s">
-        <v>28</v>
-      </c>
-      <c r="S61" s="245"/>
-      <c r="T61" s="236"/>
-      <c r="U61" s="236"/>
-      <c r="V61" s="81"/>
-      <c r="W61" s="82"/>
-      <c r="X61" s="82"/>
-      <c r="Y61" s="82"/>
-      <c r="Z61" s="82"/>
-      <c r="AA61" s="82"/>
-      <c r="AB61" s="82"/>
-      <c r="AC61" s="82"/>
-      <c r="AD61" s="82"/>
-      <c r="AE61" s="82"/>
-      <c r="AF61" s="82"/>
-      <c r="AG61" s="82"/>
-      <c r="AH61" s="82"/>
-      <c r="AI61" s="82"/>
-      <c r="AJ61" s="82"/>
-      <c r="AK61" s="82"/>
-      <c r="AL61" s="83"/>
-      <c r="AM61" s="84"/>
-      <c r="AN61" s="73"/>
-      <c r="AO61" s="71"/>
-      <c r="AP61" s="72"/>
-      <c r="AQ61" s="26"/>
-      <c r="AR61" s="27"/>
-      <c r="AS61" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT61" s="85"/>
-      <c r="AU61" s="86"/>
-      <c r="AV61" s="71"/>
-      <c r="AW61" s="72"/>
-      <c r="AX61" s="84"/>
-      <c r="AY61" s="73"/>
-      <c r="AZ61" s="71"/>
-      <c r="BA61" s="72"/>
-      <c r="BB61" s="26"/>
-      <c r="BC61" s="27"/>
-      <c r="BD61" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE61" s="85"/>
-      <c r="BF61" s="86"/>
-      <c r="BG61" s="71"/>
-      <c r="BH61" s="72"/>
+    <row r="61" spans="2:60" ht="14.4" customHeight="1">
+      <c r="B61" s="254"/>
+      <c r="C61" s="255"/>
+      <c r="D61" s="255"/>
+      <c r="E61" s="255"/>
+      <c r="F61" s="255"/>
+      <c r="G61" s="255"/>
+      <c r="H61" s="255"/>
+      <c r="I61" s="255"/>
+      <c r="J61" s="255"/>
+      <c r="K61" s="255"/>
+      <c r="L61" s="255"/>
+      <c r="M61" s="255"/>
+      <c r="N61" s="255"/>
+      <c r="O61" s="255"/>
+      <c r="P61" s="255"/>
+      <c r="Q61" s="255"/>
+      <c r="R61" s="255"/>
+      <c r="S61" s="255"/>
+      <c r="T61" s="255"/>
+      <c r="U61" s="256"/>
+      <c r="V61" s="107" t="s">
+        <v>36</v>
+      </c>
+      <c r="W61" s="108"/>
+      <c r="X61" s="108"/>
+      <c r="Y61" s="108"/>
+      <c r="Z61" s="108"/>
+      <c r="AA61" s="108"/>
+      <c r="AB61" s="108"/>
+      <c r="AC61" s="108"/>
+      <c r="AD61" s="108"/>
+      <c r="AE61" s="108"/>
+      <c r="AF61" s="108"/>
+      <c r="AG61" s="108"/>
+      <c r="AH61" s="108"/>
+      <c r="AI61" s="108"/>
+      <c r="AJ61" s="108"/>
+      <c r="AK61" s="108"/>
+      <c r="AL61" s="109"/>
+      <c r="AM61" s="77" t="s">
+        <v>48</v>
+      </c>
+      <c r="AN61" s="77"/>
+      <c r="AO61" s="24"/>
+      <c r="AP61" s="24"/>
+      <c r="AQ61" s="24"/>
+      <c r="AR61" s="24"/>
+      <c r="AS61" s="24"/>
+      <c r="AT61" s="24"/>
+      <c r="AU61" s="24"/>
+      <c r="AV61" s="24"/>
+      <c r="AW61" s="24"/>
+      <c r="AX61" s="77" t="s">
+        <v>48</v>
+      </c>
+      <c r="AY61" s="77"/>
+      <c r="AZ61" s="24"/>
+      <c r="BA61" s="24"/>
+      <c r="BB61" s="24"/>
+      <c r="BC61" s="24"/>
+      <c r="BD61" s="24"/>
+      <c r="BE61" s="24"/>
+      <c r="BF61" s="24"/>
+      <c r="BG61" s="24"/>
+      <c r="BH61" s="24"/>
     </row>
-    <row r="62" spans="2:60">
-      <c r="B62" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
-      <c r="G62" s="15"/>
-      <c r="H62" s="88"/>
-      <c r="I62" s="88"/>
-      <c r="J62" s="89"/>
-      <c r="K62" s="209" t="s">
-        <v>34</v>
-      </c>
-      <c r="L62" s="210"/>
-      <c r="M62" s="210"/>
-      <c r="N62" s="210"/>
-      <c r="O62" s="210"/>
-      <c r="P62" s="210"/>
-      <c r="Q62" s="210"/>
-      <c r="R62" s="246"/>
-      <c r="S62" s="246"/>
-      <c r="T62" s="246"/>
-      <c r="U62" s="247"/>
-      <c r="V62" s="61"/>
-      <c r="W62" s="59"/>
-      <c r="X62" s="59"/>
-      <c r="Y62" s="59"/>
-      <c r="Z62" s="59"/>
-      <c r="AA62" s="59"/>
-      <c r="AB62" s="59"/>
-      <c r="AC62" s="59"/>
-      <c r="AD62" s="59"/>
-      <c r="AE62" s="59"/>
-      <c r="AF62" s="59"/>
-      <c r="AG62" s="59"/>
-      <c r="AH62" s="59"/>
-      <c r="AI62" s="59"/>
-      <c r="AJ62" s="59"/>
-      <c r="AK62" s="59"/>
-      <c r="AL62" s="63"/>
-      <c r="AM62" s="84"/>
-      <c r="AN62" s="73"/>
-      <c r="AO62" s="71"/>
-      <c r="AP62" s="72"/>
-      <c r="AQ62" s="26"/>
-      <c r="AR62" s="27"/>
-      <c r="AS62" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT62" s="85"/>
-      <c r="AU62" s="86"/>
-      <c r="AV62" s="71"/>
-      <c r="AW62" s="72"/>
-      <c r="AX62" s="84"/>
-      <c r="AY62" s="73"/>
-      <c r="AZ62" s="71"/>
-      <c r="BA62" s="72"/>
-      <c r="BB62" s="26"/>
-      <c r="BC62" s="27"/>
-      <c r="BD62" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE62" s="85"/>
-      <c r="BF62" s="86"/>
-      <c r="BG62" s="71"/>
-      <c r="BH62" s="72"/>
+    <row r="62" spans="2:60" ht="14.4" customHeight="1">
+      <c r="B62" s="181" t="s">
+        <v>37</v>
+      </c>
+      <c r="C62" s="182"/>
+      <c r="D62" s="178" t="s">
+        <v>38</v>
+      </c>
+      <c r="E62" s="179"/>
+      <c r="F62" s="179"/>
+      <c r="G62" s="179"/>
+      <c r="H62" s="179"/>
+      <c r="I62" s="5"/>
+      <c r="J62" s="48"/>
+      <c r="K62" s="48"/>
+      <c r="L62" s="48"/>
+      <c r="M62" s="48"/>
+      <c r="N62" s="48"/>
+      <c r="O62" s="48"/>
+      <c r="P62" s="48"/>
+      <c r="Q62" s="48"/>
+      <c r="R62" s="48"/>
+      <c r="S62" s="49"/>
+      <c r="T62" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="U62" s="43"/>
+      <c r="V62" s="43"/>
+      <c r="W62" s="44"/>
+      <c r="X62" s="251"/>
+      <c r="Y62" s="252"/>
+      <c r="Z62" s="252"/>
+      <c r="AA62" s="252"/>
+      <c r="AB62" s="252"/>
+      <c r="AC62" s="253"/>
+      <c r="AD62" s="178" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE62" s="179"/>
+      <c r="AF62" s="179"/>
+      <c r="AG62" s="180"/>
+      <c r="AH62" s="108"/>
+      <c r="AI62" s="108"/>
+      <c r="AJ62" s="108"/>
+      <c r="AK62" s="108"/>
+      <c r="AL62" s="109"/>
+      <c r="AM62" s="77"/>
+      <c r="AN62" s="77"/>
+      <c r="AO62" s="24"/>
+      <c r="AP62" s="24"/>
+      <c r="AQ62" s="24"/>
+      <c r="AR62" s="24"/>
+      <c r="AS62" s="24"/>
+      <c r="AT62" s="24"/>
+      <c r="AU62" s="24"/>
+      <c r="AV62" s="24"/>
+      <c r="AW62" s="24"/>
+      <c r="AX62" s="77"/>
+      <c r="AY62" s="77"/>
+      <c r="AZ62" s="24"/>
+      <c r="BA62" s="24"/>
+      <c r="BB62" s="24"/>
+      <c r="BC62" s="24"/>
+      <c r="BD62" s="24"/>
+      <c r="BE62" s="24"/>
+      <c r="BF62" s="24"/>
+      <c r="BG62" s="24"/>
+      <c r="BH62" s="24"/>
     </row>
     <row r="63" spans="2:60">
-      <c r="B63" s="172" t="s">
-        <v>33</v>
-      </c>
-      <c r="C63" s="173"/>
-      <c r="D63" s="173"/>
-      <c r="E63" s="173"/>
-      <c r="F63" s="173"/>
-      <c r="G63" s="173"/>
-      <c r="H63" s="173"/>
-      <c r="I63" s="173"/>
-      <c r="J63" s="173"/>
-      <c r="K63" s="173"/>
-      <c r="L63" s="173"/>
-      <c r="M63" s="174"/>
-      <c r="N63" s="240" t="s">
-        <v>31</v>
-      </c>
-      <c r="O63" s="241"/>
-      <c r="P63" s="235"/>
-      <c r="Q63" s="235"/>
-      <c r="R63" s="242" t="s">
-        <v>32</v>
-      </c>
-      <c r="S63" s="243"/>
-      <c r="T63" s="237"/>
-      <c r="U63" s="237"/>
-      <c r="V63" s="61"/>
-      <c r="W63" s="258"/>
-      <c r="X63" s="258"/>
-      <c r="Y63" s="258"/>
-      <c r="Z63" s="258"/>
-      <c r="AA63" s="258"/>
-      <c r="AB63" s="258"/>
-      <c r="AC63" s="258"/>
-      <c r="AD63" s="258"/>
-      <c r="AE63" s="258"/>
-      <c r="AF63" s="59"/>
-      <c r="AG63" s="59"/>
-      <c r="AH63" s="59"/>
-      <c r="AI63" s="59"/>
-      <c r="AJ63" s="59"/>
-      <c r="AK63" s="59"/>
-      <c r="AL63" s="63"/>
-      <c r="AM63" s="84"/>
-      <c r="AN63" s="73"/>
-      <c r="AO63" s="71"/>
-      <c r="AP63" s="72"/>
-      <c r="AQ63" s="26"/>
-      <c r="AR63" s="27"/>
-      <c r="AS63" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AT63" s="85"/>
-      <c r="AU63" s="86"/>
-      <c r="AV63" s="71"/>
-      <c r="AW63" s="72"/>
-      <c r="AX63" s="84"/>
-      <c r="AY63" s="73"/>
-      <c r="AZ63" s="71"/>
-      <c r="BA63" s="72"/>
-      <c r="BB63" s="26"/>
-      <c r="BC63" s="27"/>
-      <c r="BD63" s="20" t="s">
-        <v>5</v>
-      </c>
-      <c r="BE63" s="85"/>
-      <c r="BF63" s="86"/>
-      <c r="BG63" s="71"/>
-      <c r="BH63" s="72"/>
+      <c r="B63" s="183"/>
+      <c r="C63" s="184"/>
+      <c r="D63" s="178" t="s">
+        <v>38</v>
+      </c>
+      <c r="E63" s="179"/>
+      <c r="F63" s="179"/>
+      <c r="G63" s="179"/>
+      <c r="H63" s="179"/>
+      <c r="I63" s="5"/>
+      <c r="J63" s="48"/>
+      <c r="K63" s="48"/>
+      <c r="L63" s="48"/>
+      <c r="M63" s="48"/>
+      <c r="N63" s="48"/>
+      <c r="O63" s="48"/>
+      <c r="P63" s="48"/>
+      <c r="Q63" s="48"/>
+      <c r="R63" s="48"/>
+      <c r="S63" s="49"/>
+      <c r="T63" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="U63" s="43"/>
+      <c r="V63" s="43"/>
+      <c r="W63" s="44"/>
+      <c r="X63" s="251"/>
+      <c r="Y63" s="252"/>
+      <c r="Z63" s="252"/>
+      <c r="AA63" s="252"/>
+      <c r="AB63" s="252"/>
+      <c r="AC63" s="253"/>
+      <c r="AD63" s="178" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE63" s="179"/>
+      <c r="AF63" s="179"/>
+      <c r="AG63" s="180"/>
+      <c r="AH63" s="108"/>
+      <c r="AI63" s="108"/>
+      <c r="AJ63" s="108"/>
+      <c r="AK63" s="108"/>
+      <c r="AL63" s="109"/>
+      <c r="AM63" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="AN63" s="22"/>
+      <c r="AO63" s="22"/>
+      <c r="AP63" s="22"/>
+      <c r="AQ63" s="22"/>
+      <c r="AR63" s="22"/>
+      <c r="AS63" s="22"/>
+      <c r="AT63" s="22"/>
+      <c r="AU63" s="23"/>
+      <c r="AV63" s="37"/>
+      <c r="AW63" s="37"/>
+      <c r="AX63" s="37"/>
+      <c r="AY63" s="37"/>
+      <c r="AZ63" s="37"/>
+      <c r="BA63" s="37"/>
+      <c r="BB63" s="37"/>
+      <c r="BC63" s="37"/>
+      <c r="BD63" s="37"/>
+      <c r="BE63" s="37"/>
+      <c r="BF63" s="37"/>
+      <c r="BG63" s="37"/>
+      <c r="BH63" s="110"/>
     </row>
-    <row r="64" spans="2:60">
-      <c r="B64" s="248" t="s">
-        <v>44</v>
-      </c>
-      <c r="C64" s="249"/>
-      <c r="D64" s="249"/>
-      <c r="E64" s="249"/>
-      <c r="F64" s="249"/>
-      <c r="G64" s="249"/>
-      <c r="H64" s="249"/>
-      <c r="I64" s="249"/>
-      <c r="J64" s="249"/>
-      <c r="K64" s="249"/>
-      <c r="L64" s="249"/>
-      <c r="M64" s="250"/>
-      <c r="N64" s="240" t="s">
-        <v>31</v>
-      </c>
-      <c r="O64" s="241"/>
-      <c r="P64" s="235"/>
-      <c r="Q64" s="235"/>
-      <c r="R64" s="240" t="s">
-        <v>32</v>
-      </c>
-      <c r="S64" s="241"/>
-      <c r="T64" s="235"/>
-      <c r="U64" s="235"/>
-      <c r="V64" s="62"/>
-      <c r="W64" s="60"/>
-      <c r="X64" s="60"/>
-      <c r="Y64" s="60"/>
-      <c r="Z64" s="60"/>
-      <c r="AA64" s="60"/>
-      <c r="AB64" s="60"/>
-      <c r="AC64" s="60"/>
-      <c r="AD64" s="60"/>
-      <c r="AE64" s="60"/>
-      <c r="AF64" s="60"/>
-      <c r="AG64" s="60"/>
-      <c r="AH64" s="60"/>
-      <c r="AI64" s="60"/>
-      <c r="AJ64" s="60"/>
-      <c r="AK64" s="60"/>
-      <c r="AL64" s="64"/>
-      <c r="AM64" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="AN64" s="25"/>
-      <c r="AO64" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="AP64" s="25"/>
-      <c r="AQ64" s="25"/>
-      <c r="AR64" s="25"/>
-      <c r="AS64" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="AT64" s="25"/>
-      <c r="AU64" s="25"/>
-      <c r="AV64" s="25"/>
-      <c r="AW64" s="25"/>
-      <c r="AX64" s="25" t="s">
-        <v>15</v>
-      </c>
-      <c r="AY64" s="25"/>
-      <c r="AZ64" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="BA64" s="25"/>
-      <c r="BB64" s="25"/>
-      <c r="BC64" s="25"/>
-      <c r="BD64" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="BE64" s="25"/>
-      <c r="BF64" s="25"/>
-      <c r="BG64" s="25"/>
-      <c r="BH64" s="25"/>
+    <row r="64" spans="2:60" ht="13.8">
+      <c r="B64" s="183"/>
+      <c r="C64" s="184"/>
+      <c r="D64" s="178" t="s">
+        <v>39</v>
+      </c>
+      <c r="E64" s="179"/>
+      <c r="F64" s="179"/>
+      <c r="G64" s="179"/>
+      <c r="H64" s="180"/>
+      <c r="I64" s="5"/>
+      <c r="J64" s="48"/>
+      <c r="K64" s="48"/>
+      <c r="L64" s="48"/>
+      <c r="M64" s="48"/>
+      <c r="N64" s="48"/>
+      <c r="O64" s="48"/>
+      <c r="P64" s="48"/>
+      <c r="Q64" s="48"/>
+      <c r="R64" s="48"/>
+      <c r="S64" s="49"/>
+      <c r="T64" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="U64" s="43"/>
+      <c r="V64" s="43"/>
+      <c r="W64" s="44"/>
+      <c r="X64" s="251"/>
+      <c r="Y64" s="252"/>
+      <c r="Z64" s="252"/>
+      <c r="AA64" s="252"/>
+      <c r="AB64" s="252"/>
+      <c r="AC64" s="253"/>
+      <c r="AD64" s="178" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE64" s="179"/>
+      <c r="AF64" s="179"/>
+      <c r="AG64" s="180"/>
+      <c r="AH64" s="108"/>
+      <c r="AI64" s="108"/>
+      <c r="AJ64" s="108"/>
+      <c r="AK64" s="108"/>
+      <c r="AL64" s="109"/>
+      <c r="AM64" s="45" t="s">
+        <v>50</v>
+      </c>
+      <c r="AN64" s="46"/>
+      <c r="AO64" s="46"/>
+      <c r="AP64" s="46"/>
+      <c r="AQ64" s="46"/>
+      <c r="AR64" s="94"/>
+      <c r="AS64" s="95"/>
+      <c r="AT64" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AU64" s="96"/>
+      <c r="AV64" s="97"/>
+      <c r="AW64" s="93" t="s">
+        <v>51</v>
+      </c>
+      <c r="AX64" s="93"/>
+      <c r="AY64" s="93"/>
+      <c r="AZ64" s="93"/>
+      <c r="BA64" s="93"/>
+      <c r="BB64" s="93"/>
+      <c r="BC64" s="93"/>
+      <c r="BD64" s="94"/>
+      <c r="BE64" s="95"/>
+      <c r="BF64" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="BG64" s="96"/>
+      <c r="BH64" s="97"/>
     </row>
-    <row r="65" spans="2:60" ht="14.4" customHeight="1">
-      <c r="B65" s="254"/>
-      <c r="C65" s="255"/>
-      <c r="D65" s="255"/>
-      <c r="E65" s="255"/>
-      <c r="F65" s="255"/>
-      <c r="G65" s="255"/>
-      <c r="H65" s="255"/>
-      <c r="I65" s="255"/>
-      <c r="J65" s="255"/>
-      <c r="K65" s="255"/>
-      <c r="L65" s="255"/>
-      <c r="M65" s="255"/>
-      <c r="N65" s="255"/>
-      <c r="O65" s="255"/>
-      <c r="P65" s="255"/>
-      <c r="Q65" s="255"/>
-      <c r="R65" s="255"/>
-      <c r="S65" s="255"/>
-      <c r="T65" s="255"/>
-      <c r="U65" s="256"/>
-      <c r="V65" s="107" t="s">
-        <v>36</v>
-      </c>
-      <c r="W65" s="108"/>
-      <c r="X65" s="108"/>
-      <c r="Y65" s="108"/>
-      <c r="Z65" s="108"/>
-      <c r="AA65" s="108"/>
-      <c r="AB65" s="108"/>
-      <c r="AC65" s="108"/>
-      <c r="AD65" s="108"/>
-      <c r="AE65" s="108"/>
-      <c r="AF65" s="108"/>
-      <c r="AG65" s="108"/>
+    <row r="65" spans="2:60" ht="13.8">
+      <c r="B65" s="183"/>
+      <c r="C65" s="184"/>
+      <c r="D65" s="178" t="s">
+        <v>40</v>
+      </c>
+      <c r="E65" s="179"/>
+      <c r="F65" s="179"/>
+      <c r="G65" s="179"/>
+      <c r="H65" s="180"/>
+      <c r="I65" s="5"/>
+      <c r="J65" s="48"/>
+      <c r="K65" s="48"/>
+      <c r="L65" s="48"/>
+      <c r="M65" s="48"/>
+      <c r="N65" s="48"/>
+      <c r="O65" s="48"/>
+      <c r="P65" s="48"/>
+      <c r="Q65" s="48"/>
+      <c r="R65" s="48"/>
+      <c r="S65" s="49"/>
+      <c r="T65" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="U65" s="43"/>
+      <c r="V65" s="43"/>
+      <c r="W65" s="44"/>
+      <c r="X65" s="251"/>
+      <c r="Y65" s="252"/>
+      <c r="Z65" s="252"/>
+      <c r="AA65" s="252"/>
+      <c r="AB65" s="252"/>
+      <c r="AC65" s="253"/>
+      <c r="AD65" s="74" t="s">
+        <v>56</v>
+      </c>
+      <c r="AE65" s="75"/>
+      <c r="AF65" s="75"/>
+      <c r="AG65" s="257"/>
       <c r="AH65" s="108"/>
       <c r="AI65" s="108"/>
       <c r="AJ65" s="108"/>
       <c r="AK65" s="108"/>
       <c r="AL65" s="109"/>
-      <c r="AM65" s="77" t="s">
-        <v>48</v>
-      </c>
-      <c r="AN65" s="77"/>
-      <c r="AO65" s="24"/>
-      <c r="AP65" s="24"/>
-      <c r="AQ65" s="24"/>
-      <c r="AR65" s="24"/>
-      <c r="AS65" s="24"/>
-      <c r="AT65" s="24"/>
-      <c r="AU65" s="24"/>
-      <c r="AV65" s="24"/>
-      <c r="AW65" s="24"/>
-      <c r="AX65" s="77" t="s">
-        <v>48</v>
-      </c>
-      <c r="AY65" s="77"/>
-      <c r="AZ65" s="24"/>
-      <c r="BA65" s="24"/>
-      <c r="BB65" s="24"/>
-      <c r="BC65" s="24"/>
-      <c r="BD65" s="24"/>
-      <c r="BE65" s="24"/>
-      <c r="BF65" s="24"/>
-      <c r="BG65" s="24"/>
-      <c r="BH65" s="24"/>
+      <c r="AM65" s="107" t="s">
+        <v>49</v>
+      </c>
+      <c r="AN65" s="108"/>
+      <c r="AO65" s="108"/>
+      <c r="AP65" s="108"/>
+      <c r="AQ65" s="108"/>
+      <c r="AR65" s="114"/>
+      <c r="AS65" s="114"/>
+      <c r="AT65" s="115"/>
+      <c r="AU65" s="115"/>
+      <c r="AV65" s="115"/>
+      <c r="AW65" s="115"/>
+      <c r="AX65" s="115"/>
+      <c r="AY65" s="115"/>
+      <c r="AZ65" s="115"/>
+      <c r="BA65" s="115"/>
+      <c r="BB65" s="115"/>
+      <c r="BC65" s="115"/>
+      <c r="BD65" s="114"/>
+      <c r="BE65" s="114"/>
+      <c r="BF65" s="115"/>
+      <c r="BG65" s="115"/>
+      <c r="BH65" s="116"/>
     </row>
-    <row r="66" spans="2:60" ht="14.4" customHeight="1">
-      <c r="B66" s="181" t="s">
-        <v>37</v>
-      </c>
-      <c r="C66" s="182"/>
+    <row r="66" spans="2:60">
+      <c r="B66" s="185"/>
+      <c r="C66" s="186"/>
       <c r="D66" s="178" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E66" s="179"/>
       <c r="F66" s="179"/>
       <c r="G66" s="179"/>
-      <c r="H66" s="179"/>
+      <c r="H66" s="180"/>
       <c r="I66" s="5"/>
       <c r="J66" s="48"/>
       <c r="K66" s="48"/>
@@ -6228,517 +6248,216 @@
       <c r="Q66" s="48"/>
       <c r="R66" s="48"/>
       <c r="S66" s="49"/>
-      <c r="T66" s="42" t="s">
+      <c r="T66" s="45" t="s">
         <v>42</v>
       </c>
-      <c r="U66" s="43"/>
-      <c r="V66" s="43"/>
-      <c r="W66" s="44"/>
+      <c r="U66" s="46"/>
+      <c r="V66" s="46"/>
+      <c r="W66" s="47"/>
       <c r="X66" s="251"/>
       <c r="Y66" s="252"/>
       <c r="Z66" s="252"/>
       <c r="AA66" s="252"/>
       <c r="AB66" s="252"/>
       <c r="AC66" s="253"/>
-      <c r="AD66" s="178" t="s">
+      <c r="AD66" s="74" t="s">
         <v>56</v>
       </c>
-      <c r="AE66" s="179"/>
-      <c r="AF66" s="179"/>
-      <c r="AG66" s="180"/>
+      <c r="AE66" s="75"/>
+      <c r="AF66" s="75"/>
+      <c r="AG66" s="257"/>
       <c r="AH66" s="108"/>
       <c r="AI66" s="108"/>
       <c r="AJ66" s="108"/>
       <c r="AK66" s="108"/>
       <c r="AL66" s="109"/>
-      <c r="AM66" s="77"/>
-      <c r="AN66" s="77"/>
-      <c r="AO66" s="24"/>
-      <c r="AP66" s="24"/>
-      <c r="AQ66" s="24"/>
-      <c r="AR66" s="24"/>
-      <c r="AS66" s="24"/>
-      <c r="AT66" s="24"/>
-      <c r="AU66" s="24"/>
-      <c r="AV66" s="24"/>
-      <c r="AW66" s="24"/>
-      <c r="AX66" s="77"/>
-      <c r="AY66" s="77"/>
-      <c r="AZ66" s="24"/>
-      <c r="BA66" s="24"/>
-      <c r="BB66" s="24"/>
-      <c r="BC66" s="24"/>
-      <c r="BD66" s="24"/>
-      <c r="BE66" s="24"/>
-      <c r="BF66" s="24"/>
-      <c r="BG66" s="24"/>
-      <c r="BH66" s="24"/>
+      <c r="AM66" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="AN66" s="37"/>
+      <c r="AO66" s="37"/>
+      <c r="AP66" s="37"/>
+      <c r="AQ66" s="37"/>
+      <c r="AR66" s="34"/>
+      <c r="AS66" s="34"/>
+      <c r="AT66" s="34"/>
+      <c r="AU66" s="34"/>
+      <c r="AV66" s="34"/>
+      <c r="AW66" s="34"/>
+      <c r="AX66" s="34"/>
+      <c r="AY66" s="34"/>
+      <c r="AZ66" s="34"/>
+      <c r="BA66" s="34"/>
+      <c r="BB66" s="34"/>
+      <c r="BC66" s="34"/>
+      <c r="BD66" s="34"/>
+      <c r="BE66" s="34"/>
+      <c r="BF66" s="34"/>
+      <c r="BG66" s="34"/>
+      <c r="BH66" s="35"/>
     </row>
     <row r="67" spans="2:60">
-      <c r="B67" s="183"/>
-      <c r="C67" s="184"/>
-      <c r="D67" s="178" t="s">
-        <v>38</v>
-      </c>
-      <c r="E67" s="179"/>
-      <c r="F67" s="179"/>
-      <c r="G67" s="179"/>
-      <c r="H67" s="179"/>
-      <c r="I67" s="5"/>
-      <c r="J67" s="48"/>
-      <c r="K67" s="48"/>
-      <c r="L67" s="48"/>
-      <c r="M67" s="48"/>
-      <c r="N67" s="48"/>
-      <c r="O67" s="48"/>
-      <c r="P67" s="48"/>
-      <c r="Q67" s="48"/>
-      <c r="R67" s="48"/>
-      <c r="S67" s="49"/>
-      <c r="T67" s="42" t="s">
-        <v>42</v>
-      </c>
-      <c r="U67" s="43"/>
-      <c r="V67" s="43"/>
-      <c r="W67" s="44"/>
-      <c r="X67" s="251"/>
-      <c r="Y67" s="252"/>
-      <c r="Z67" s="252"/>
-      <c r="AA67" s="252"/>
-      <c r="AB67" s="252"/>
-      <c r="AC67" s="253"/>
-      <c r="AD67" s="178" t="s">
-        <v>56</v>
-      </c>
-      <c r="AE67" s="179"/>
-      <c r="AF67" s="179"/>
-      <c r="AG67" s="180"/>
-      <c r="AH67" s="108"/>
-      <c r="AI67" s="108"/>
-      <c r="AJ67" s="108"/>
-      <c r="AK67" s="108"/>
-      <c r="AL67" s="109"/>
-      <c r="AM67" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="AN67" s="22"/>
-      <c r="AO67" s="22"/>
-      <c r="AP67" s="22"/>
-      <c r="AQ67" s="22"/>
-      <c r="AR67" s="22"/>
-      <c r="AS67" s="22"/>
-      <c r="AT67" s="22"/>
-      <c r="AU67" s="23"/>
-      <c r="AV67" s="37"/>
-      <c r="AW67" s="37"/>
-      <c r="AX67" s="37"/>
-      <c r="AY67" s="37"/>
-      <c r="AZ67" s="37"/>
-      <c r="BA67" s="37"/>
-      <c r="BB67" s="37"/>
-      <c r="BC67" s="37"/>
-      <c r="BD67" s="37"/>
-      <c r="BE67" s="37"/>
-      <c r="BF67" s="37"/>
-      <c r="BG67" s="37"/>
-      <c r="BH67" s="110"/>
-    </row>
-    <row r="68" spans="2:60" ht="13.8">
-      <c r="B68" s="183"/>
-      <c r="C68" s="184"/>
-      <c r="D68" s="178" t="s">
-        <v>39</v>
-      </c>
-      <c r="E68" s="179"/>
-      <c r="F68" s="179"/>
-      <c r="G68" s="179"/>
-      <c r="H68" s="180"/>
-      <c r="I68" s="5"/>
-      <c r="J68" s="48"/>
-      <c r="K68" s="48"/>
-      <c r="L68" s="48"/>
-      <c r="M68" s="48"/>
-      <c r="N68" s="48"/>
-      <c r="O68" s="48"/>
-      <c r="P68" s="48"/>
-      <c r="Q68" s="48"/>
-      <c r="R68" s="48"/>
-      <c r="S68" s="49"/>
-      <c r="T68" s="42" t="s">
-        <v>42</v>
-      </c>
-      <c r="U68" s="43"/>
-      <c r="V68" s="43"/>
-      <c r="W68" s="44"/>
-      <c r="X68" s="251"/>
-      <c r="Y68" s="252"/>
-      <c r="Z68" s="252"/>
-      <c r="AA68" s="252"/>
-      <c r="AB68" s="252"/>
-      <c r="AC68" s="253"/>
-      <c r="AD68" s="178" t="s">
-        <v>56</v>
-      </c>
-      <c r="AE68" s="179"/>
-      <c r="AF68" s="179"/>
-      <c r="AG68" s="180"/>
-      <c r="AH68" s="108"/>
-      <c r="AI68" s="108"/>
-      <c r="AJ68" s="108"/>
-      <c r="AK68" s="108"/>
-      <c r="AL68" s="109"/>
-      <c r="AM68" s="45" t="s">
-        <v>50</v>
-      </c>
-      <c r="AN68" s="46"/>
-      <c r="AO68" s="46"/>
-      <c r="AP68" s="46"/>
-      <c r="AQ68" s="46"/>
-      <c r="AR68" s="94"/>
-      <c r="AS68" s="95"/>
-      <c r="AT68" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="AU68" s="96"/>
-      <c r="AV68" s="97"/>
-      <c r="AW68" s="93" t="s">
-        <v>51</v>
-      </c>
-      <c r="AX68" s="93"/>
-      <c r="AY68" s="93"/>
-      <c r="AZ68" s="93"/>
-      <c r="BA68" s="93"/>
-      <c r="BB68" s="93"/>
-      <c r="BC68" s="93"/>
-      <c r="BD68" s="94"/>
-      <c r="BE68" s="95"/>
-      <c r="BF68" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="BG68" s="96"/>
-      <c r="BH68" s="97"/>
-    </row>
-    <row r="69" spans="2:60" ht="13.8">
-      <c r="B69" s="183"/>
-      <c r="C69" s="184"/>
-      <c r="D69" s="178" t="s">
-        <v>40</v>
-      </c>
-      <c r="E69" s="179"/>
-      <c r="F69" s="179"/>
-      <c r="G69" s="179"/>
-      <c r="H69" s="180"/>
-      <c r="I69" s="5"/>
-      <c r="J69" s="48"/>
-      <c r="K69" s="48"/>
-      <c r="L69" s="48"/>
-      <c r="M69" s="48"/>
-      <c r="N69" s="48"/>
-      <c r="O69" s="48"/>
-      <c r="P69" s="48"/>
-      <c r="Q69" s="48"/>
-      <c r="R69" s="48"/>
-      <c r="S69" s="49"/>
-      <c r="T69" s="42" t="s">
-        <v>42</v>
-      </c>
-      <c r="U69" s="43"/>
-      <c r="V69" s="43"/>
-      <c r="W69" s="44"/>
-      <c r="X69" s="251"/>
-      <c r="Y69" s="252"/>
-      <c r="Z69" s="252"/>
-      <c r="AA69" s="252"/>
-      <c r="AB69" s="252"/>
-      <c r="AC69" s="253"/>
-      <c r="AD69" s="74" t="s">
-        <v>56</v>
-      </c>
-      <c r="AE69" s="75"/>
-      <c r="AF69" s="75"/>
-      <c r="AG69" s="257"/>
-      <c r="AH69" s="108"/>
-      <c r="AI69" s="108"/>
-      <c r="AJ69" s="108"/>
-      <c r="AK69" s="108"/>
-      <c r="AL69" s="109"/>
-      <c r="AM69" s="107" t="s">
-        <v>49</v>
-      </c>
-      <c r="AN69" s="108"/>
-      <c r="AO69" s="108"/>
-      <c r="AP69" s="108"/>
-      <c r="AQ69" s="108"/>
-      <c r="AR69" s="114"/>
-      <c r="AS69" s="114"/>
-      <c r="AT69" s="115"/>
-      <c r="AU69" s="115"/>
-      <c r="AV69" s="115"/>
-      <c r="AW69" s="115"/>
-      <c r="AX69" s="115"/>
-      <c r="AY69" s="115"/>
-      <c r="AZ69" s="115"/>
-      <c r="BA69" s="115"/>
-      <c r="BB69" s="115"/>
-      <c r="BC69" s="115"/>
-      <c r="BD69" s="114"/>
-      <c r="BE69" s="114"/>
-      <c r="BF69" s="115"/>
-      <c r="BG69" s="115"/>
-      <c r="BH69" s="116"/>
-    </row>
-    <row r="70" spans="2:60">
-      <c r="B70" s="185"/>
-      <c r="C70" s="186"/>
-      <c r="D70" s="178" t="s">
-        <v>41</v>
-      </c>
-      <c r="E70" s="179"/>
-      <c r="F70" s="179"/>
-      <c r="G70" s="179"/>
-      <c r="H70" s="180"/>
-      <c r="I70" s="5"/>
-      <c r="J70" s="48"/>
-      <c r="K70" s="48"/>
-      <c r="L70" s="48"/>
-      <c r="M70" s="48"/>
-      <c r="N70" s="48"/>
-      <c r="O70" s="48"/>
-      <c r="P70" s="48"/>
-      <c r="Q70" s="48"/>
-      <c r="R70" s="48"/>
-      <c r="S70" s="49"/>
-      <c r="T70" s="45" t="s">
-        <v>42</v>
-      </c>
-      <c r="U70" s="46"/>
-      <c r="V70" s="46"/>
-      <c r="W70" s="47"/>
-      <c r="X70" s="251"/>
-      <c r="Y70" s="252"/>
-      <c r="Z70" s="252"/>
-      <c r="AA70" s="252"/>
-      <c r="AB70" s="252"/>
-      <c r="AC70" s="253"/>
-      <c r="AD70" s="74" t="s">
-        <v>56</v>
-      </c>
-      <c r="AE70" s="75"/>
-      <c r="AF70" s="75"/>
-      <c r="AG70" s="257"/>
-      <c r="AH70" s="108"/>
-      <c r="AI70" s="108"/>
-      <c r="AJ70" s="108"/>
-      <c r="AK70" s="108"/>
-      <c r="AL70" s="109"/>
-      <c r="AM70" s="36" t="s">
-        <v>57</v>
-      </c>
-      <c r="AN70" s="37"/>
-      <c r="AO70" s="37"/>
-      <c r="AP70" s="37"/>
-      <c r="AQ70" s="37"/>
-      <c r="AR70" s="34"/>
-      <c r="AS70" s="34"/>
-      <c r="AT70" s="34"/>
-      <c r="AU70" s="34"/>
-      <c r="AV70" s="34"/>
-      <c r="AW70" s="34"/>
-      <c r="AX70" s="34"/>
-      <c r="AY70" s="34"/>
-      <c r="AZ70" s="34"/>
-      <c r="BA70" s="34"/>
-      <c r="BB70" s="34"/>
-      <c r="BC70" s="34"/>
-      <c r="BD70" s="34"/>
-      <c r="BE70" s="34"/>
-      <c r="BF70" s="34"/>
-      <c r="BG70" s="34"/>
-      <c r="BH70" s="35"/>
-    </row>
-    <row r="71" spans="2:60">
-      <c r="B71" s="209" t="s">
+      <c r="B67" s="209" t="s">
         <v>58</v>
       </c>
-      <c r="C71" s="210"/>
-      <c r="D71" s="210"/>
-      <c r="E71" s="210"/>
-      <c r="F71" s="210"/>
-      <c r="G71" s="210"/>
-      <c r="H71" s="210"/>
-      <c r="I71" s="210"/>
-      <c r="J71" s="210"/>
-      <c r="K71" s="210"/>
-      <c r="L71" s="210"/>
-      <c r="M71" s="210"/>
-      <c r="N71" s="210"/>
-      <c r="O71" s="210"/>
-      <c r="P71" s="210"/>
-      <c r="Q71" s="210"/>
-      <c r="R71" s="210"/>
-      <c r="S71" s="210"/>
-      <c r="T71" s="210"/>
-      <c r="U71" s="210"/>
-      <c r="V71" s="210"/>
-      <c r="W71" s="210"/>
-      <c r="X71" s="210"/>
-      <c r="Y71" s="210"/>
-      <c r="Z71" s="210"/>
-      <c r="AA71" s="210"/>
-      <c r="AB71" s="210"/>
-      <c r="AC71" s="210"/>
-      <c r="AD71" s="210"/>
-      <c r="AE71" s="210"/>
-      <c r="AF71" s="210"/>
-      <c r="AG71" s="210"/>
-      <c r="AH71" s="210"/>
-      <c r="AI71" s="210"/>
-      <c r="AJ71" s="210"/>
-      <c r="AK71" s="210"/>
-      <c r="AL71" s="210"/>
-      <c r="AM71" s="210"/>
-      <c r="AN71" s="210"/>
-      <c r="AO71" s="210"/>
-      <c r="AP71" s="210"/>
-      <c r="AQ71" s="210"/>
-      <c r="AR71" s="210"/>
-      <c r="AS71" s="210"/>
-      <c r="AT71" s="210"/>
-      <c r="AU71" s="210"/>
-      <c r="AV71" s="210"/>
-      <c r="AW71" s="210"/>
-      <c r="AX71" s="210"/>
-      <c r="AY71" s="210"/>
-      <c r="AZ71" s="210"/>
-      <c r="BA71" s="210"/>
-      <c r="BB71" s="210"/>
-      <c r="BC71" s="210"/>
-      <c r="BD71" s="210"/>
-      <c r="BE71" s="210"/>
-      <c r="BF71" s="210"/>
-      <c r="BG71" s="210"/>
-      <c r="BH71" s="211"/>
+      <c r="C67" s="210"/>
+      <c r="D67" s="210"/>
+      <c r="E67" s="210"/>
+      <c r="F67" s="210"/>
+      <c r="G67" s="210"/>
+      <c r="H67" s="210"/>
+      <c r="I67" s="210"/>
+      <c r="J67" s="210"/>
+      <c r="K67" s="210"/>
+      <c r="L67" s="210"/>
+      <c r="M67" s="210"/>
+      <c r="N67" s="210"/>
+      <c r="O67" s="210"/>
+      <c r="P67" s="210"/>
+      <c r="Q67" s="210"/>
+      <c r="R67" s="210"/>
+      <c r="S67" s="210"/>
+      <c r="T67" s="210"/>
+      <c r="U67" s="210"/>
+      <c r="V67" s="210"/>
+      <c r="W67" s="210"/>
+      <c r="X67" s="210"/>
+      <c r="Y67" s="210"/>
+      <c r="Z67" s="210"/>
+      <c r="AA67" s="210"/>
+      <c r="AB67" s="210"/>
+      <c r="AC67" s="210"/>
+      <c r="AD67" s="210"/>
+      <c r="AE67" s="210"/>
+      <c r="AF67" s="210"/>
+      <c r="AG67" s="210"/>
+      <c r="AH67" s="210"/>
+      <c r="AI67" s="210"/>
+      <c r="AJ67" s="210"/>
+      <c r="AK67" s="210"/>
+      <c r="AL67" s="210"/>
+      <c r="AM67" s="210"/>
+      <c r="AN67" s="210"/>
+      <c r="AO67" s="210"/>
+      <c r="AP67" s="210"/>
+      <c r="AQ67" s="210"/>
+      <c r="AR67" s="210"/>
+      <c r="AS67" s="210"/>
+      <c r="AT67" s="210"/>
+      <c r="AU67" s="210"/>
+      <c r="AV67" s="210"/>
+      <c r="AW67" s="210"/>
+      <c r="AX67" s="210"/>
+      <c r="AY67" s="210"/>
+      <c r="AZ67" s="210"/>
+      <c r="BA67" s="210"/>
+      <c r="BB67" s="210"/>
+      <c r="BC67" s="210"/>
+      <c r="BD67" s="210"/>
+      <c r="BE67" s="210"/>
+      <c r="BF67" s="210"/>
+      <c r="BG67" s="210"/>
+      <c r="BH67" s="211"/>
     </row>
   </sheetData>
-  <mergeCells count="1074">
-    <mergeCell ref="AV67:BH67"/>
-    <mergeCell ref="AG53:AI53"/>
-    <mergeCell ref="AJ53:AL53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="D54:Q54"/>
-    <mergeCell ref="AZ61:BA61"/>
-    <mergeCell ref="AZ62:BA62"/>
-    <mergeCell ref="AZ63:BA63"/>
-    <mergeCell ref="AQ62:AR62"/>
-    <mergeCell ref="AQ60:AR60"/>
-    <mergeCell ref="AT60:AU60"/>
-    <mergeCell ref="BB60:BC60"/>
-    <mergeCell ref="BE60:BF60"/>
-    <mergeCell ref="AZ60:BA60"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="E58:G58"/>
-    <mergeCell ref="H58:J58"/>
-    <mergeCell ref="BG58:BH58"/>
-    <mergeCell ref="B65:U65"/>
-    <mergeCell ref="V65:AL65"/>
-    <mergeCell ref="D66:H66"/>
-    <mergeCell ref="D67:H67"/>
-    <mergeCell ref="V63:AE64"/>
-    <mergeCell ref="AF63:AL64"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="D52:Q52"/>
-    <mergeCell ref="R52:S52"/>
-    <mergeCell ref="T52:U52"/>
-    <mergeCell ref="B49:C49"/>
+  <mergeCells count="994">
+    <mergeCell ref="AV63:BH63"/>
+    <mergeCell ref="AZ57:BA57"/>
+    <mergeCell ref="AZ58:BA58"/>
+    <mergeCell ref="AZ59:BA59"/>
+    <mergeCell ref="AQ58:AR58"/>
+    <mergeCell ref="AQ56:AR56"/>
+    <mergeCell ref="AT56:AU56"/>
+    <mergeCell ref="BB56:BC56"/>
+    <mergeCell ref="BE56:BF56"/>
+    <mergeCell ref="AZ56:BA56"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="E54:G54"/>
+    <mergeCell ref="H54:J54"/>
+    <mergeCell ref="BG54:BH54"/>
+    <mergeCell ref="B61:U61"/>
+    <mergeCell ref="V61:AL61"/>
+    <mergeCell ref="D62:H62"/>
+    <mergeCell ref="D63:H63"/>
+    <mergeCell ref="V59:AE60"/>
+    <mergeCell ref="AF59:AL60"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="D50:Q50"/>
+    <mergeCell ref="R50:S50"/>
+    <mergeCell ref="T50:U50"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="D47:Q47"/>
+    <mergeCell ref="R47:S47"/>
+    <mergeCell ref="T47:U47"/>
+    <mergeCell ref="AH62:AL62"/>
+    <mergeCell ref="AH63:AL63"/>
+    <mergeCell ref="AH64:AL64"/>
+    <mergeCell ref="AH65:AL65"/>
+    <mergeCell ref="AH66:AL66"/>
+    <mergeCell ref="X62:AC62"/>
+    <mergeCell ref="X63:AC63"/>
+    <mergeCell ref="X64:AC64"/>
+    <mergeCell ref="X65:AC65"/>
+    <mergeCell ref="X66:AC66"/>
+    <mergeCell ref="P59:Q59"/>
+    <mergeCell ref="P60:Q60"/>
+    <mergeCell ref="T57:U57"/>
+    <mergeCell ref="T59:U59"/>
+    <mergeCell ref="T60:U60"/>
+    <mergeCell ref="N57:O57"/>
+    <mergeCell ref="N59:O59"/>
+    <mergeCell ref="N60:O60"/>
+    <mergeCell ref="R59:S59"/>
+    <mergeCell ref="R60:S60"/>
+    <mergeCell ref="R57:S57"/>
+    <mergeCell ref="R58:U58"/>
+    <mergeCell ref="K58:Q58"/>
+    <mergeCell ref="B60:M60"/>
+    <mergeCell ref="AG8:AH8"/>
+    <mergeCell ref="AI8:AL8"/>
+    <mergeCell ref="L51:Q51"/>
+    <mergeCell ref="S51:X51"/>
+    <mergeCell ref="Z51:AE51"/>
+    <mergeCell ref="AG51:AL51"/>
+    <mergeCell ref="K53:Q53"/>
+    <mergeCell ref="R53:X53"/>
+    <mergeCell ref="Y53:AE53"/>
+    <mergeCell ref="AF53:AL53"/>
+    <mergeCell ref="K28:Q28"/>
+    <mergeCell ref="R28:X28"/>
+    <mergeCell ref="Y28:AE28"/>
+    <mergeCell ref="AF28:AL28"/>
+    <mergeCell ref="K52:Q52"/>
+    <mergeCell ref="R52:X52"/>
     <mergeCell ref="D49:Q49"/>
     <mergeCell ref="R49:S49"/>
     <mergeCell ref="T49:U49"/>
-    <mergeCell ref="AH66:AL66"/>
-    <mergeCell ref="AH67:AL67"/>
-    <mergeCell ref="AH68:AL68"/>
-    <mergeCell ref="AH69:AL69"/>
-    <mergeCell ref="AH70:AL70"/>
-    <mergeCell ref="X66:AC66"/>
-    <mergeCell ref="X67:AC67"/>
-    <mergeCell ref="X68:AC68"/>
-    <mergeCell ref="X69:AC69"/>
-    <mergeCell ref="X70:AC70"/>
-    <mergeCell ref="P63:Q63"/>
-    <mergeCell ref="P64:Q64"/>
-    <mergeCell ref="T61:U61"/>
-    <mergeCell ref="T63:U63"/>
-    <mergeCell ref="T64:U64"/>
-    <mergeCell ref="N61:O61"/>
-    <mergeCell ref="N63:O63"/>
-    <mergeCell ref="N64:O64"/>
-    <mergeCell ref="R63:S63"/>
-    <mergeCell ref="R64:S64"/>
-    <mergeCell ref="R61:S61"/>
-    <mergeCell ref="R62:U62"/>
-    <mergeCell ref="K62:Q62"/>
-    <mergeCell ref="B64:M64"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="D53:Q53"/>
-    <mergeCell ref="R53:S53"/>
-    <mergeCell ref="T53:U53"/>
-    <mergeCell ref="R54:S54"/>
-    <mergeCell ref="T54:U54"/>
-    <mergeCell ref="AG8:AH8"/>
-    <mergeCell ref="AI8:AL8"/>
-    <mergeCell ref="L55:Q55"/>
-    <mergeCell ref="S55:X55"/>
-    <mergeCell ref="Z55:AE55"/>
-    <mergeCell ref="AG55:AL55"/>
-    <mergeCell ref="K57:Q57"/>
-    <mergeCell ref="R57:X57"/>
-    <mergeCell ref="Y57:AE57"/>
-    <mergeCell ref="AF57:AL57"/>
-    <mergeCell ref="K30:Q30"/>
-    <mergeCell ref="R30:X30"/>
-    <mergeCell ref="Y30:AE30"/>
-    <mergeCell ref="AF30:AL30"/>
-    <mergeCell ref="K56:Q56"/>
-    <mergeCell ref="R56:X56"/>
-    <mergeCell ref="D51:Q51"/>
-    <mergeCell ref="R51:S51"/>
-    <mergeCell ref="T51:U51"/>
-    <mergeCell ref="V49:W49"/>
-    <mergeCell ref="X49:Z49"/>
-    <mergeCell ref="AA49:AC49"/>
-    <mergeCell ref="AD49:AF49"/>
-    <mergeCell ref="AA48:AC48"/>
-    <mergeCell ref="AD48:AF48"/>
-    <mergeCell ref="P32:Q32"/>
-    <mergeCell ref="R32:S32"/>
-    <mergeCell ref="T32:V32"/>
-    <mergeCell ref="W32:X32"/>
+    <mergeCell ref="V47:W47"/>
+    <mergeCell ref="X47:Z47"/>
+    <mergeCell ref="AA47:AC47"/>
+    <mergeCell ref="AD47:AF47"/>
+    <mergeCell ref="AA46:AC46"/>
+    <mergeCell ref="AD46:AF46"/>
+    <mergeCell ref="P30:Q30"/>
+    <mergeCell ref="R30:S30"/>
+    <mergeCell ref="T30:V30"/>
+    <mergeCell ref="W30:X30"/>
     <mergeCell ref="T24:U24"/>
     <mergeCell ref="T25:U25"/>
     <mergeCell ref="X22:Z22"/>
     <mergeCell ref="AJ18:AL18"/>
     <mergeCell ref="AJ11:AL11"/>
     <mergeCell ref="V25:W25"/>
-    <mergeCell ref="AV59:AW59"/>
-    <mergeCell ref="AX59:AY59"/>
-    <mergeCell ref="AQ59:AR59"/>
-    <mergeCell ref="AT59:AU59"/>
-    <mergeCell ref="V53:W53"/>
-    <mergeCell ref="X53:Z53"/>
-    <mergeCell ref="AA53:AC53"/>
-    <mergeCell ref="AD53:AF53"/>
-    <mergeCell ref="V54:W54"/>
-    <mergeCell ref="X54:Z54"/>
-    <mergeCell ref="AA54:AC54"/>
-    <mergeCell ref="V52:W52"/>
-    <mergeCell ref="X52:Z52"/>
-    <mergeCell ref="AA52:AC52"/>
-    <mergeCell ref="AD52:AF52"/>
+    <mergeCell ref="AV55:AW55"/>
+    <mergeCell ref="AX55:AY55"/>
     <mergeCell ref="AQ55:AR55"/>
     <mergeCell ref="AT55:AU55"/>
-    <mergeCell ref="AM28:AN28"/>
-    <mergeCell ref="AO28:AP28"/>
-    <mergeCell ref="AV28:AW28"/>
-    <mergeCell ref="AX28:AY28"/>
+    <mergeCell ref="V50:W50"/>
+    <mergeCell ref="X50:Z50"/>
+    <mergeCell ref="AA50:AC50"/>
+    <mergeCell ref="AD50:AF50"/>
+    <mergeCell ref="AQ51:AR51"/>
+    <mergeCell ref="AT51:AU51"/>
     <mergeCell ref="AM25:AN25"/>
     <mergeCell ref="AO25:AP25"/>
     <mergeCell ref="AV25:AW25"/>
@@ -6746,137 +6465,95 @@
     <mergeCell ref="AQ25:AR25"/>
     <mergeCell ref="AT25:AU25"/>
     <mergeCell ref="AT18:AU18"/>
-    <mergeCell ref="AI32:AJ32"/>
-    <mergeCell ref="AK32:AL32"/>
-    <mergeCell ref="AG52:AI52"/>
-    <mergeCell ref="AJ52:AL52"/>
-    <mergeCell ref="AG49:AI49"/>
-    <mergeCell ref="AJ49:AL49"/>
-    <mergeCell ref="AG48:AI48"/>
-    <mergeCell ref="AJ48:AL48"/>
-    <mergeCell ref="AG37:AI37"/>
-    <mergeCell ref="AJ37:AL37"/>
-    <mergeCell ref="AJ36:AL36"/>
+    <mergeCell ref="AI30:AJ30"/>
+    <mergeCell ref="AK30:AL30"/>
+    <mergeCell ref="AG50:AI50"/>
+    <mergeCell ref="AJ50:AL50"/>
+    <mergeCell ref="AG47:AI47"/>
+    <mergeCell ref="AJ47:AL47"/>
+    <mergeCell ref="AG46:AI46"/>
+    <mergeCell ref="AJ46:AL46"/>
+    <mergeCell ref="AG35:AI35"/>
+    <mergeCell ref="AJ35:AL35"/>
+    <mergeCell ref="AJ34:AL34"/>
     <mergeCell ref="AG19:AI19"/>
     <mergeCell ref="AJ19:AL19"/>
-    <mergeCell ref="AJ38:AL38"/>
-    <mergeCell ref="AG27:AI27"/>
+    <mergeCell ref="AJ36:AL36"/>
     <mergeCell ref="AG22:AI22"/>
-    <mergeCell ref="AJ28:AL28"/>
-    <mergeCell ref="BE59:BF59"/>
-    <mergeCell ref="AZ59:BA59"/>
-    <mergeCell ref="AQ58:AR58"/>
-    <mergeCell ref="AT58:AU58"/>
-    <mergeCell ref="BB58:BC58"/>
-    <mergeCell ref="AJ54:AL54"/>
-    <mergeCell ref="AG29:AL29"/>
-    <mergeCell ref="AF31:AL31"/>
-    <mergeCell ref="AD36:AF36"/>
-    <mergeCell ref="AJ51:AL51"/>
+    <mergeCell ref="BE55:BF55"/>
+    <mergeCell ref="AZ55:BA55"/>
+    <mergeCell ref="AQ54:AR54"/>
+    <mergeCell ref="AT54:AU54"/>
+    <mergeCell ref="BB54:BC54"/>
+    <mergeCell ref="AG27:AL27"/>
+    <mergeCell ref="AF29:AL29"/>
+    <mergeCell ref="AD34:AF34"/>
+    <mergeCell ref="AJ49:AL49"/>
     <mergeCell ref="AM4:BH5"/>
     <mergeCell ref="AR1:AY1"/>
     <mergeCell ref="AZ1:BH1"/>
     <mergeCell ref="AR2:BH2"/>
     <mergeCell ref="B3:R3"/>
     <mergeCell ref="B6:R6"/>
-    <mergeCell ref="BE58:BF58"/>
-    <mergeCell ref="AZ58:BA58"/>
-    <mergeCell ref="AT56:AU57"/>
-    <mergeCell ref="AV56:AW57"/>
-    <mergeCell ref="AX56:AY57"/>
-    <mergeCell ref="AZ56:BA57"/>
-    <mergeCell ref="BB56:BC57"/>
-    <mergeCell ref="BD56:BD57"/>
-    <mergeCell ref="BE56:BF57"/>
-    <mergeCell ref="BG56:BH57"/>
-    <mergeCell ref="AV58:AW58"/>
-    <mergeCell ref="AM56:AN57"/>
-    <mergeCell ref="AO56:AP57"/>
-    <mergeCell ref="AQ56:AR57"/>
-    <mergeCell ref="AS56:AS57"/>
-    <mergeCell ref="AQ54:AR54"/>
-    <mergeCell ref="AT54:AU54"/>
+    <mergeCell ref="BE54:BF54"/>
+    <mergeCell ref="AZ54:BA54"/>
+    <mergeCell ref="AT52:AU53"/>
+    <mergeCell ref="AV52:AW53"/>
+    <mergeCell ref="AX52:AY53"/>
+    <mergeCell ref="AZ52:BA53"/>
+    <mergeCell ref="BB52:BC53"/>
+    <mergeCell ref="BD52:BD53"/>
+    <mergeCell ref="BE52:BF53"/>
+    <mergeCell ref="BG52:BH53"/>
+    <mergeCell ref="AV54:AW54"/>
+    <mergeCell ref="AM52:AN53"/>
+    <mergeCell ref="AO52:AP53"/>
+    <mergeCell ref="AQ52:AR53"/>
+    <mergeCell ref="AS52:AS53"/>
     <mergeCell ref="Q1:AQ2"/>
-    <mergeCell ref="BE54:BF54"/>
-    <mergeCell ref="BB55:BC55"/>
-    <mergeCell ref="BE55:BF55"/>
-    <mergeCell ref="AZ54:BA54"/>
-    <mergeCell ref="AZ55:BA55"/>
-    <mergeCell ref="AM58:AN58"/>
-    <mergeCell ref="AO58:AP58"/>
-    <mergeCell ref="AX58:AY58"/>
-    <mergeCell ref="B71:BH71"/>
+    <mergeCell ref="BB51:BC51"/>
+    <mergeCell ref="BE51:BF51"/>
+    <mergeCell ref="AZ51:BA51"/>
+    <mergeCell ref="AM54:AN54"/>
+    <mergeCell ref="AO54:AP54"/>
+    <mergeCell ref="AX54:AY54"/>
+    <mergeCell ref="B67:BH67"/>
     <mergeCell ref="AA8:AB8"/>
     <mergeCell ref="AC8:AF8"/>
-    <mergeCell ref="AM68:AQ68"/>
-    <mergeCell ref="AM65:AN66"/>
-    <mergeCell ref="AM64:AN64"/>
-    <mergeCell ref="BG63:BH63"/>
-    <mergeCell ref="AM63:AN63"/>
-    <mergeCell ref="E35:U35"/>
+    <mergeCell ref="AM64:AQ64"/>
+    <mergeCell ref="AM61:AN62"/>
+    <mergeCell ref="AM60:AN60"/>
     <mergeCell ref="BG59:BH59"/>
-    <mergeCell ref="AM60:AN60"/>
-    <mergeCell ref="AO60:AP60"/>
-    <mergeCell ref="AV60:AW60"/>
-    <mergeCell ref="AX60:AY60"/>
-    <mergeCell ref="BG60:BH60"/>
     <mergeCell ref="AM59:AN59"/>
-    <mergeCell ref="AO59:AP59"/>
-    <mergeCell ref="AA58:AC58"/>
-    <mergeCell ref="AD58:AE58"/>
-    <mergeCell ref="AF58:AH58"/>
-    <mergeCell ref="AI58:AJ58"/>
-    <mergeCell ref="AK58:AL58"/>
-    <mergeCell ref="BG54:BH54"/>
+    <mergeCell ref="E33:U33"/>
+    <mergeCell ref="BG55:BH55"/>
+    <mergeCell ref="AM56:AN56"/>
+    <mergeCell ref="AO56:AP56"/>
+    <mergeCell ref="AV56:AW56"/>
+    <mergeCell ref="AX56:AY56"/>
+    <mergeCell ref="BG56:BH56"/>
     <mergeCell ref="AM55:AN55"/>
     <mergeCell ref="AO55:AP55"/>
-    <mergeCell ref="AV55:AW55"/>
-    <mergeCell ref="AX55:AY55"/>
-    <mergeCell ref="BG55:BH55"/>
-    <mergeCell ref="AM54:AN54"/>
-    <mergeCell ref="AO54:AP54"/>
-    <mergeCell ref="AV54:AW54"/>
-    <mergeCell ref="AX54:AY54"/>
-    <mergeCell ref="BG52:BH52"/>
-    <mergeCell ref="AM53:AN53"/>
-    <mergeCell ref="AO53:AP53"/>
-    <mergeCell ref="AV53:AW53"/>
-    <mergeCell ref="AX53:AY53"/>
-    <mergeCell ref="BG53:BH53"/>
-    <mergeCell ref="AM52:AN52"/>
-    <mergeCell ref="AO52:AP52"/>
-    <mergeCell ref="AV52:AW52"/>
-    <mergeCell ref="AX52:AY52"/>
-    <mergeCell ref="AQ52:AR52"/>
-    <mergeCell ref="AT52:AU52"/>
-    <mergeCell ref="AQ53:AR53"/>
-    <mergeCell ref="AT53:AU53"/>
-    <mergeCell ref="BB52:BC52"/>
-    <mergeCell ref="BE52:BF52"/>
-    <mergeCell ref="BB53:BC53"/>
-    <mergeCell ref="BE53:BF53"/>
-    <mergeCell ref="AZ52:BA52"/>
-    <mergeCell ref="AZ53:BA53"/>
-    <mergeCell ref="BG50:BH50"/>
+    <mergeCell ref="AA54:AC54"/>
+    <mergeCell ref="AD54:AE54"/>
+    <mergeCell ref="AF54:AH54"/>
+    <mergeCell ref="AI54:AJ54"/>
+    <mergeCell ref="AK54:AL54"/>
     <mergeCell ref="AM51:AN51"/>
     <mergeCell ref="AO51:AP51"/>
     <mergeCell ref="AV51:AW51"/>
     <mergeCell ref="AX51:AY51"/>
     <mergeCell ref="BG51:BH51"/>
+    <mergeCell ref="BG50:BH50"/>
     <mergeCell ref="AM50:AN50"/>
     <mergeCell ref="AO50:AP50"/>
     <mergeCell ref="AV50:AW50"/>
     <mergeCell ref="AX50:AY50"/>
     <mergeCell ref="AQ50:AR50"/>
     <mergeCell ref="AT50:AU50"/>
-    <mergeCell ref="AQ51:AR51"/>
-    <mergeCell ref="AT51:AU51"/>
     <mergeCell ref="BB50:BC50"/>
     <mergeCell ref="BE50:BF50"/>
-    <mergeCell ref="BB51:BC51"/>
-    <mergeCell ref="BE51:BF51"/>
     <mergeCell ref="AZ50:BA50"/>
-    <mergeCell ref="AZ51:BA51"/>
     <mergeCell ref="BG48:BH48"/>
     <mergeCell ref="AM49:AN49"/>
     <mergeCell ref="AO49:AP49"/>
@@ -7057,43 +6734,48 @@
     <mergeCell ref="BE33:BF33"/>
     <mergeCell ref="AZ32:BA32"/>
     <mergeCell ref="AZ33:BA33"/>
-    <mergeCell ref="BG29:BH29"/>
-    <mergeCell ref="AM29:AN29"/>
-    <mergeCell ref="AO29:AP29"/>
-    <mergeCell ref="AV29:AW29"/>
-    <mergeCell ref="AX29:AY29"/>
-    <mergeCell ref="AQ29:AR29"/>
-    <mergeCell ref="AT29:AU29"/>
-    <mergeCell ref="BB29:BC29"/>
-    <mergeCell ref="BE29:BF29"/>
-    <mergeCell ref="AZ29:BA29"/>
-    <mergeCell ref="AM30:AN31"/>
-    <mergeCell ref="AO30:AP31"/>
-    <mergeCell ref="AQ30:AR31"/>
-    <mergeCell ref="AS30:AS31"/>
-    <mergeCell ref="AT30:AU31"/>
-    <mergeCell ref="AV30:AW31"/>
-    <mergeCell ref="AX30:AY31"/>
-    <mergeCell ref="AZ30:BA31"/>
-    <mergeCell ref="BB30:BC31"/>
-    <mergeCell ref="BD30:BD31"/>
-    <mergeCell ref="BE30:BF31"/>
-    <mergeCell ref="BG30:BH31"/>
-    <mergeCell ref="BG28:BH28"/>
+    <mergeCell ref="BG30:BH30"/>
+    <mergeCell ref="AM31:AN31"/>
+    <mergeCell ref="AO31:AP31"/>
+    <mergeCell ref="AV31:AW31"/>
+    <mergeCell ref="AX31:AY31"/>
+    <mergeCell ref="BG31:BH31"/>
+    <mergeCell ref="AM30:AN30"/>
+    <mergeCell ref="AO30:AP30"/>
+    <mergeCell ref="AV30:AW30"/>
+    <mergeCell ref="AX30:AY30"/>
+    <mergeCell ref="AQ30:AR30"/>
+    <mergeCell ref="AT30:AU30"/>
+    <mergeCell ref="AQ31:AR31"/>
+    <mergeCell ref="AT31:AU31"/>
+    <mergeCell ref="BB30:BC30"/>
+    <mergeCell ref="BE30:BF30"/>
+    <mergeCell ref="BB31:BC31"/>
+    <mergeCell ref="BE31:BF31"/>
+    <mergeCell ref="AZ30:BA30"/>
+    <mergeCell ref="AZ31:BA31"/>
+    <mergeCell ref="BG27:BH27"/>
     <mergeCell ref="AM27:AN27"/>
     <mergeCell ref="AO27:AP27"/>
     <mergeCell ref="AV27:AW27"/>
     <mergeCell ref="AX27:AY27"/>
     <mergeCell ref="AQ27:AR27"/>
     <mergeCell ref="AT27:AU27"/>
-    <mergeCell ref="AQ28:AR28"/>
-    <mergeCell ref="AT28:AU28"/>
     <mergeCell ref="BB27:BC27"/>
     <mergeCell ref="BE27:BF27"/>
-    <mergeCell ref="BB28:BC28"/>
-    <mergeCell ref="BE28:BF28"/>
     <mergeCell ref="AZ27:BA27"/>
-    <mergeCell ref="AZ28:BA28"/>
+    <mergeCell ref="AM28:AN29"/>
+    <mergeCell ref="AO28:AP29"/>
+    <mergeCell ref="AQ28:AR29"/>
+    <mergeCell ref="AS28:AS29"/>
+    <mergeCell ref="AT28:AU29"/>
+    <mergeCell ref="AV28:AW29"/>
+    <mergeCell ref="AX28:AY29"/>
+    <mergeCell ref="AZ28:BA29"/>
+    <mergeCell ref="BB28:BC29"/>
+    <mergeCell ref="BD28:BD29"/>
+    <mergeCell ref="BE28:BF29"/>
+    <mergeCell ref="BG28:BH29"/>
     <mergeCell ref="AM26:AN26"/>
     <mergeCell ref="AO26:AP26"/>
     <mergeCell ref="AV26:AW26"/>
@@ -7102,7 +6784,6 @@
     <mergeCell ref="AQ26:AR26"/>
     <mergeCell ref="AT26:AU26"/>
     <mergeCell ref="BE26:BF26"/>
-    <mergeCell ref="BG27:BH27"/>
     <mergeCell ref="BB26:BC26"/>
     <mergeCell ref="AZ26:BA26"/>
     <mergeCell ref="BG23:BH23"/>
@@ -7160,10 +6841,10 @@
     <mergeCell ref="AZ22:BA22"/>
     <mergeCell ref="BB22:BC22"/>
     <mergeCell ref="AZ20:BA20"/>
-    <mergeCell ref="D68:H68"/>
-    <mergeCell ref="D69:H69"/>
-    <mergeCell ref="D70:H70"/>
-    <mergeCell ref="B66:C70"/>
+    <mergeCell ref="D64:H64"/>
+    <mergeCell ref="D65:H65"/>
+    <mergeCell ref="D66:H66"/>
+    <mergeCell ref="B62:C66"/>
     <mergeCell ref="AV16:AW16"/>
     <mergeCell ref="AX16:AY16"/>
     <mergeCell ref="BG16:BH16"/>
@@ -7188,62 +6869,44 @@
     <mergeCell ref="AQ17:AR17"/>
     <mergeCell ref="AT17:AU17"/>
     <mergeCell ref="AQ18:AR18"/>
-    <mergeCell ref="B63:M63"/>
-    <mergeCell ref="K59:Q60"/>
-    <mergeCell ref="AD54:AF54"/>
-    <mergeCell ref="AG54:AI54"/>
-    <mergeCell ref="H62:J62"/>
-    <mergeCell ref="K58:L58"/>
-    <mergeCell ref="M58:O58"/>
-    <mergeCell ref="P58:Q58"/>
-    <mergeCell ref="R58:S58"/>
-    <mergeCell ref="T58:V58"/>
-    <mergeCell ref="W58:X58"/>
-    <mergeCell ref="Y58:Z58"/>
-    <mergeCell ref="C55:F55"/>
-    <mergeCell ref="G55:J57"/>
-    <mergeCell ref="B56:F56"/>
-    <mergeCell ref="B57:F57"/>
-    <mergeCell ref="R59:X60"/>
-    <mergeCell ref="Y59:AE60"/>
-    <mergeCell ref="AF59:AL60"/>
-    <mergeCell ref="B61:M61"/>
-    <mergeCell ref="B59:J60"/>
-    <mergeCell ref="Y56:AE56"/>
-    <mergeCell ref="AF56:AL56"/>
-    <mergeCell ref="P61:Q61"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="D50:Q50"/>
-    <mergeCell ref="R50:S50"/>
-    <mergeCell ref="T50:U50"/>
-    <mergeCell ref="V50:W50"/>
-    <mergeCell ref="X50:Z50"/>
-    <mergeCell ref="AA50:AC50"/>
-    <mergeCell ref="AD50:AF50"/>
-    <mergeCell ref="AG50:AI50"/>
-    <mergeCell ref="AJ50:AL50"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="AG51:AI51"/>
-    <mergeCell ref="V51:W51"/>
-    <mergeCell ref="X51:Z51"/>
-    <mergeCell ref="AA51:AC51"/>
-    <mergeCell ref="AD51:AF51"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="D47:Q47"/>
-    <mergeCell ref="R47:S47"/>
-    <mergeCell ref="T47:U47"/>
-    <mergeCell ref="V47:W47"/>
-    <mergeCell ref="X47:Z47"/>
-    <mergeCell ref="AA47:AC47"/>
-    <mergeCell ref="AD47:AF47"/>
-    <mergeCell ref="AG47:AI47"/>
-    <mergeCell ref="AJ47:AL47"/>
+    <mergeCell ref="B59:M59"/>
+    <mergeCell ref="K55:Q56"/>
+    <mergeCell ref="H58:J58"/>
+    <mergeCell ref="K54:L54"/>
+    <mergeCell ref="M54:O54"/>
+    <mergeCell ref="P54:Q54"/>
+    <mergeCell ref="R54:S54"/>
+    <mergeCell ref="T54:V54"/>
+    <mergeCell ref="W54:X54"/>
+    <mergeCell ref="Y54:Z54"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="G51:J53"/>
+    <mergeCell ref="B52:F52"/>
+    <mergeCell ref="B53:F53"/>
+    <mergeCell ref="R55:X56"/>
+    <mergeCell ref="Y55:AE56"/>
+    <mergeCell ref="AF55:AL56"/>
+    <mergeCell ref="B57:M57"/>
+    <mergeCell ref="B55:J56"/>
+    <mergeCell ref="Y52:AE52"/>
+    <mergeCell ref="AF52:AL52"/>
+    <mergeCell ref="P57:Q57"/>
     <mergeCell ref="B48:C48"/>
     <mergeCell ref="D48:Q48"/>
     <mergeCell ref="R48:S48"/>
     <mergeCell ref="T48:U48"/>
     <mergeCell ref="V48:W48"/>
     <mergeCell ref="X48:Z48"/>
+    <mergeCell ref="AA48:AC48"/>
+    <mergeCell ref="AD48:AF48"/>
+    <mergeCell ref="AG48:AI48"/>
+    <mergeCell ref="AJ48:AL48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="AG49:AI49"/>
+    <mergeCell ref="V49:W49"/>
+    <mergeCell ref="X49:Z49"/>
+    <mergeCell ref="AA49:AC49"/>
+    <mergeCell ref="AD49:AF49"/>
     <mergeCell ref="B45:C45"/>
     <mergeCell ref="D45:Q45"/>
     <mergeCell ref="R45:S45"/>
@@ -7260,10 +6923,6 @@
     <mergeCell ref="T46:U46"/>
     <mergeCell ref="V46:W46"/>
     <mergeCell ref="X46:Z46"/>
-    <mergeCell ref="AA46:AC46"/>
-    <mergeCell ref="AD46:AF46"/>
-    <mergeCell ref="AG46:AI46"/>
-    <mergeCell ref="AJ46:AL46"/>
     <mergeCell ref="B43:C43"/>
     <mergeCell ref="D43:Q43"/>
     <mergeCell ref="R43:S43"/>
@@ -7324,6 +6983,26 @@
     <mergeCell ref="AD40:AF40"/>
     <mergeCell ref="AG40:AI40"/>
     <mergeCell ref="AJ40:AL40"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="D37:Q37"/>
+    <mergeCell ref="R37:S37"/>
+    <mergeCell ref="T37:U37"/>
+    <mergeCell ref="V37:W37"/>
+    <mergeCell ref="X37:Z37"/>
+    <mergeCell ref="AA37:AC37"/>
+    <mergeCell ref="AD37:AF37"/>
+    <mergeCell ref="AG37:AI37"/>
+    <mergeCell ref="AJ37:AL37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D38:Q38"/>
+    <mergeCell ref="R38:S38"/>
+    <mergeCell ref="T38:U38"/>
+    <mergeCell ref="V38:W38"/>
+    <mergeCell ref="X38:Z38"/>
+    <mergeCell ref="AA38:AC38"/>
+    <mergeCell ref="AD38:AF38"/>
+    <mergeCell ref="AG38:AI38"/>
+    <mergeCell ref="AJ38:AL38"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
@@ -7335,14 +7014,9 @@
     <mergeCell ref="AD15:AF15"/>
     <mergeCell ref="AD24:AF24"/>
     <mergeCell ref="AA18:AC18"/>
-    <mergeCell ref="X27:Z27"/>
-    <mergeCell ref="AA27:AC27"/>
-    <mergeCell ref="AD27:AF27"/>
     <mergeCell ref="X23:Z23"/>
     <mergeCell ref="AA23:AC23"/>
     <mergeCell ref="AD23:AF23"/>
-    <mergeCell ref="T27:U27"/>
-    <mergeCell ref="V27:W27"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="T12:U12"/>
@@ -7356,31 +7030,17 @@
     <mergeCell ref="AD14:AF14"/>
     <mergeCell ref="T26:U26"/>
     <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="D37:Q37"/>
-    <mergeCell ref="R37:S37"/>
-    <mergeCell ref="T37:U37"/>
-    <mergeCell ref="V37:W37"/>
-    <mergeCell ref="AG36:AI36"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="H32:J32"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="M32:O32"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:Q38"/>
-    <mergeCell ref="R38:S38"/>
-    <mergeCell ref="T38:U38"/>
-    <mergeCell ref="V38:W38"/>
-    <mergeCell ref="X38:Z38"/>
-    <mergeCell ref="AA38:AC38"/>
-    <mergeCell ref="AD38:AF38"/>
-    <mergeCell ref="AG38:AI38"/>
-    <mergeCell ref="B33:J34"/>
-    <mergeCell ref="K33:Q34"/>
-    <mergeCell ref="R33:X34"/>
-    <mergeCell ref="Y33:AE34"/>
-    <mergeCell ref="AF33:AL34"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:Q35"/>
+    <mergeCell ref="R35:S35"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="V35:W35"/>
+    <mergeCell ref="AG34:AI34"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="M30:O30"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="D36:Q36"/>
     <mergeCell ref="R36:S36"/>
@@ -7388,28 +7048,37 @@
     <mergeCell ref="V36:W36"/>
     <mergeCell ref="X36:Z36"/>
     <mergeCell ref="AA36:AC36"/>
+    <mergeCell ref="AD36:AF36"/>
+    <mergeCell ref="AG36:AI36"/>
+    <mergeCell ref="B31:J32"/>
+    <mergeCell ref="K31:Q32"/>
+    <mergeCell ref="R31:X32"/>
+    <mergeCell ref="Y31:AE32"/>
+    <mergeCell ref="AF31:AL32"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D34:Q34"/>
+    <mergeCell ref="R34:S34"/>
+    <mergeCell ref="T34:U34"/>
+    <mergeCell ref="V34:W34"/>
+    <mergeCell ref="X34:Z34"/>
+    <mergeCell ref="AA34:AC34"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="AD32:AE32"/>
-    <mergeCell ref="AF32:AH32"/>
-    <mergeCell ref="AA28:AC28"/>
-    <mergeCell ref="AD28:AF28"/>
-    <mergeCell ref="AG28:AI28"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="AD30:AE30"/>
+    <mergeCell ref="AF30:AH30"/>
     <mergeCell ref="X25:Z25"/>
     <mergeCell ref="AA25:AC25"/>
     <mergeCell ref="AD25:AF25"/>
     <mergeCell ref="AG25:AI25"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="G29:J31"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="G27:J29"/>
     <mergeCell ref="X26:Z26"/>
-    <mergeCell ref="Y32:Z32"/>
-    <mergeCell ref="AA32:AC32"/>
+    <mergeCell ref="Y30:Z30"/>
+    <mergeCell ref="AA30:AC30"/>
     <mergeCell ref="AG14:AI14"/>
     <mergeCell ref="AJ14:AL14"/>
     <mergeCell ref="AD20:AF20"/>
@@ -7448,8 +7117,6 @@
     <mergeCell ref="D24:Q24"/>
     <mergeCell ref="D25:Q25"/>
     <mergeCell ref="D26:Q26"/>
-    <mergeCell ref="D27:Q27"/>
-    <mergeCell ref="D28:Q28"/>
     <mergeCell ref="D17:Q17"/>
     <mergeCell ref="D18:Q18"/>
     <mergeCell ref="D19:Q19"/>
@@ -7462,13 +7129,10 @@
     <mergeCell ref="D14:Q14"/>
     <mergeCell ref="D15:Q15"/>
     <mergeCell ref="D16:Q16"/>
-    <mergeCell ref="V28:W28"/>
     <mergeCell ref="T23:U23"/>
     <mergeCell ref="D10:Q10"/>
     <mergeCell ref="T17:U17"/>
     <mergeCell ref="R26:S26"/>
-    <mergeCell ref="R27:S27"/>
-    <mergeCell ref="R28:S28"/>
     <mergeCell ref="R17:S17"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="B10:C10"/>
@@ -7542,18 +7206,17 @@
     <mergeCell ref="V9:AL9"/>
     <mergeCell ref="AA11:AC11"/>
     <mergeCell ref="AD11:AF11"/>
-    <mergeCell ref="AT62:AU62"/>
-    <mergeCell ref="AQ63:AR63"/>
+    <mergeCell ref="AT58:AU58"/>
+    <mergeCell ref="AQ59:AR59"/>
     <mergeCell ref="B1:P2"/>
-    <mergeCell ref="L29:Q29"/>
-    <mergeCell ref="K31:Q31"/>
-    <mergeCell ref="S29:X29"/>
-    <mergeCell ref="R31:X31"/>
-    <mergeCell ref="Z29:AE29"/>
-    <mergeCell ref="Y31:AE31"/>
-    <mergeCell ref="AT63:AU63"/>
+    <mergeCell ref="L27:Q27"/>
+    <mergeCell ref="K29:Q29"/>
+    <mergeCell ref="S27:X27"/>
+    <mergeCell ref="R29:X29"/>
+    <mergeCell ref="Z27:AE27"/>
+    <mergeCell ref="Y29:AE29"/>
+    <mergeCell ref="AT59:AU59"/>
     <mergeCell ref="BB15:BC15"/>
-    <mergeCell ref="T28:U28"/>
     <mergeCell ref="AH3:AL3"/>
     <mergeCell ref="AH4:AL4"/>
     <mergeCell ref="AH5:AL5"/>
@@ -7570,44 +7233,44 @@
     <mergeCell ref="V4:Z4"/>
     <mergeCell ref="BE15:BF15"/>
     <mergeCell ref="BB16:BC16"/>
-    <mergeCell ref="BD64:BH64"/>
+    <mergeCell ref="BD60:BH60"/>
     <mergeCell ref="AH7:AL7"/>
-    <mergeCell ref="AR68:AS68"/>
-    <mergeCell ref="AU68:AV68"/>
-    <mergeCell ref="AO64:AR64"/>
-    <mergeCell ref="AO65:AR66"/>
-    <mergeCell ref="AM69:AQ69"/>
-    <mergeCell ref="AR69:BH69"/>
-    <mergeCell ref="BB61:BC61"/>
-    <mergeCell ref="BE61:BF61"/>
-    <mergeCell ref="BB62:BC62"/>
-    <mergeCell ref="BE62:BF62"/>
-    <mergeCell ref="BB63:BC63"/>
-    <mergeCell ref="BE63:BF63"/>
-    <mergeCell ref="AO63:AP63"/>
-    <mergeCell ref="AV63:AW63"/>
-    <mergeCell ref="AX63:AY63"/>
-    <mergeCell ref="BG61:BH61"/>
-    <mergeCell ref="AM62:AN62"/>
-    <mergeCell ref="AO62:AP62"/>
-    <mergeCell ref="AV62:AW62"/>
-    <mergeCell ref="AX62:AY62"/>
-    <mergeCell ref="BG62:BH62"/>
+    <mergeCell ref="AR64:AS64"/>
+    <mergeCell ref="AU64:AV64"/>
+    <mergeCell ref="AO60:AR60"/>
+    <mergeCell ref="AO61:AR62"/>
+    <mergeCell ref="AM65:AQ65"/>
+    <mergeCell ref="AR65:BH65"/>
+    <mergeCell ref="BB57:BC57"/>
+    <mergeCell ref="BE57:BF57"/>
+    <mergeCell ref="BB58:BC58"/>
+    <mergeCell ref="BE58:BF58"/>
+    <mergeCell ref="BB59:BC59"/>
+    <mergeCell ref="BE59:BF59"/>
+    <mergeCell ref="AO59:AP59"/>
+    <mergeCell ref="AV59:AW59"/>
+    <mergeCell ref="AX59:AY59"/>
+    <mergeCell ref="BG57:BH57"/>
+    <mergeCell ref="AM58:AN58"/>
+    <mergeCell ref="AO58:AP58"/>
+    <mergeCell ref="AV58:AW58"/>
+    <mergeCell ref="AX58:AY58"/>
+    <mergeCell ref="BG58:BH58"/>
     <mergeCell ref="BG11:BH11"/>
     <mergeCell ref="BE16:BF16"/>
     <mergeCell ref="BB17:BC17"/>
-    <mergeCell ref="AX64:AY64"/>
+    <mergeCell ref="AX60:AY60"/>
     <mergeCell ref="BE17:BF17"/>
-    <mergeCell ref="AZ64:BC64"/>
+    <mergeCell ref="AZ60:BC60"/>
     <mergeCell ref="AJ12:AL12"/>
     <mergeCell ref="AG21:AI21"/>
     <mergeCell ref="AJ21:AL21"/>
     <mergeCell ref="X10:Z10"/>
     <mergeCell ref="V10:W10"/>
-    <mergeCell ref="AW68:BC68"/>
-    <mergeCell ref="BD68:BE68"/>
-    <mergeCell ref="BG68:BH68"/>
-    <mergeCell ref="T66:W66"/>
+    <mergeCell ref="AW64:BC64"/>
+    <mergeCell ref="BD64:BE64"/>
+    <mergeCell ref="BG64:BH64"/>
+    <mergeCell ref="T62:W62"/>
     <mergeCell ref="AZ10:BF10"/>
     <mergeCell ref="AZ11:BF11"/>
     <mergeCell ref="AM6:AP7"/>
@@ -7635,8 +7298,8 @@
     <mergeCell ref="AH6:AL6"/>
     <mergeCell ref="T10:U10"/>
     <mergeCell ref="AO16:AP16"/>
-    <mergeCell ref="AS65:AW66"/>
-    <mergeCell ref="AX65:AY66"/>
+    <mergeCell ref="AS61:AW62"/>
+    <mergeCell ref="AX61:AY62"/>
     <mergeCell ref="AJ13:AL13"/>
     <mergeCell ref="AD12:AF12"/>
     <mergeCell ref="AD17:AF17"/>
@@ -7645,56 +7308,53 @@
     <mergeCell ref="AD21:AF21"/>
     <mergeCell ref="AJ22:AL22"/>
     <mergeCell ref="AG18:AI18"/>
-    <mergeCell ref="V61:AL61"/>
-    <mergeCell ref="V62:AL62"/>
-    <mergeCell ref="AM61:AN61"/>
-    <mergeCell ref="AO61:AP61"/>
-    <mergeCell ref="AJ27:AL27"/>
-    <mergeCell ref="X28:Z28"/>
-    <mergeCell ref="AV61:AW61"/>
-    <mergeCell ref="AX61:AY61"/>
-    <mergeCell ref="AQ61:AR61"/>
-    <mergeCell ref="AT61:AU61"/>
+    <mergeCell ref="V57:AL57"/>
+    <mergeCell ref="V58:AL58"/>
+    <mergeCell ref="AM57:AN57"/>
+    <mergeCell ref="AO57:AP57"/>
+    <mergeCell ref="AV57:AW57"/>
+    <mergeCell ref="AX57:AY57"/>
+    <mergeCell ref="AQ57:AR57"/>
+    <mergeCell ref="AT57:AU57"/>
     <mergeCell ref="AG20:AI20"/>
-    <mergeCell ref="V35:AL35"/>
+    <mergeCell ref="V33:AL33"/>
     <mergeCell ref="AG13:AI13"/>
     <mergeCell ref="AG26:AI26"/>
     <mergeCell ref="AJ26:AL26"/>
     <mergeCell ref="AG23:AI23"/>
     <mergeCell ref="AJ23:AL23"/>
     <mergeCell ref="AD13:AF13"/>
-    <mergeCell ref="X37:Z37"/>
-    <mergeCell ref="AA37:AC37"/>
-    <mergeCell ref="AD37:AF37"/>
-    <mergeCell ref="AZ65:BC66"/>
-    <mergeCell ref="BD65:BH66"/>
-    <mergeCell ref="AS64:AW64"/>
-    <mergeCell ref="BB54:BC54"/>
-    <mergeCell ref="BB59:BC59"/>
+    <mergeCell ref="X35:Z35"/>
+    <mergeCell ref="AA35:AC35"/>
+    <mergeCell ref="AD35:AF35"/>
+    <mergeCell ref="AZ61:BC62"/>
+    <mergeCell ref="BD61:BH62"/>
+    <mergeCell ref="AS60:AW60"/>
+    <mergeCell ref="BB55:BC55"/>
     <mergeCell ref="AZ12:BA14"/>
-    <mergeCell ref="AR70:BH70"/>
-    <mergeCell ref="AM70:AQ70"/>
+    <mergeCell ref="AR66:BH66"/>
+    <mergeCell ref="AM66:AQ66"/>
     <mergeCell ref="D4:R5"/>
     <mergeCell ref="D7:R8"/>
-    <mergeCell ref="T67:W67"/>
-    <mergeCell ref="T68:W68"/>
-    <mergeCell ref="T69:W69"/>
-    <mergeCell ref="T70:W70"/>
+    <mergeCell ref="T63:W63"/>
+    <mergeCell ref="T64:W64"/>
+    <mergeCell ref="T65:W65"/>
+    <mergeCell ref="T66:W66"/>
+    <mergeCell ref="J62:S62"/>
+    <mergeCell ref="J63:S63"/>
+    <mergeCell ref="J64:S64"/>
+    <mergeCell ref="J65:S65"/>
     <mergeCell ref="J66:S66"/>
-    <mergeCell ref="J67:S67"/>
-    <mergeCell ref="J68:S68"/>
-    <mergeCell ref="J69:S69"/>
-    <mergeCell ref="J70:S70"/>
     <mergeCell ref="AQ12:AU14"/>
     <mergeCell ref="AV12:AW14"/>
     <mergeCell ref="AX12:AY14"/>
     <mergeCell ref="BG15:BH15"/>
     <mergeCell ref="AM16:AN16"/>
+    <mergeCell ref="AD62:AG62"/>
+    <mergeCell ref="AD63:AG63"/>
+    <mergeCell ref="AD64:AG64"/>
+    <mergeCell ref="AD65:AG65"/>
     <mergeCell ref="AD66:AG66"/>
-    <mergeCell ref="AD67:AG67"/>
-    <mergeCell ref="AD68:AG68"/>
-    <mergeCell ref="AD69:AG69"/>
-    <mergeCell ref="AD70:AG70"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="9.3503937007874127E-3" right="0.19685039370078741" top="0.31496062992125984" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
protokół z kategoriami i w ogóle
</commit_message>
<xml_diff>
--- a/app/templates/protocol_template.xlsx
+++ b/app/templates/protocol_template.xlsx
@@ -2384,11 +2384,11 @@
         <v>20</v>
       </c>
       <c r="C9" s="108"/>
-      <c r="D9" s="108"/>
-      <c r="E9" s="146">
+      <c r="D9" s="146">
         <f>D4</f>
         <v>0</v>
       </c>
+      <c r="E9" s="146"/>
       <c r="F9" s="146"/>
       <c r="G9" s="146"/>
       <c r="H9" s="146"/>
@@ -3990,11 +3990,11 @@
         <v>27</v>
       </c>
       <c r="C33" s="108"/>
-      <c r="D33" s="108"/>
-      <c r="E33" s="146">
+      <c r="D33" s="146">
         <f>D7</f>
         <v>0</v>
       </c>
+      <c r="E33" s="146"/>
       <c r="F33" s="146"/>
       <c r="G33" s="146"/>
       <c r="H33" s="146"/>
@@ -6525,7 +6525,7 @@
     <mergeCell ref="AM60:AN60"/>
     <mergeCell ref="BG59:BH59"/>
     <mergeCell ref="AM59:AN59"/>
-    <mergeCell ref="E33:U33"/>
+    <mergeCell ref="D33:U33"/>
     <mergeCell ref="BG55:BH55"/>
     <mergeCell ref="AM56:AN56"/>
     <mergeCell ref="AO56:AP56"/>
@@ -7065,7 +7065,7 @@
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B33:C33"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="AD30:AE30"/>
@@ -7134,7 +7134,7 @@
     <mergeCell ref="T17:U17"/>
     <mergeCell ref="R26:S26"/>
     <mergeCell ref="R17:S17"/>
-    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="X14:Z14"/>
@@ -7152,7 +7152,7 @@
     <mergeCell ref="AJ20:AL20"/>
     <mergeCell ref="X17:Z17"/>
     <mergeCell ref="AG11:AI11"/>
-    <mergeCell ref="E9:U9"/>
+    <mergeCell ref="D9:U9"/>
     <mergeCell ref="AJ10:AL10"/>
     <mergeCell ref="AG10:AI10"/>
     <mergeCell ref="AD10:AF10"/>

</xml_diff>